<commit_message>
CASM-5723 - Update CANU to support bare-metal fabric manager
</commit_message>
<xml_diff>
--- a/tests/data/Full_Architecture_Golden_Config_1.1.5.xlsx
+++ b/tests/data/Full_Architecture_Golden_Config_1.1.5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasbates/canu-container/canu/tests/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cspiller/tickets/CASM-5723/canu_src/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100FBE82-86D9-0640-A3A1-B346532A1D08}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A2A660-5375-DF41-AE22-FD8859523E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="78080" yWindow="2140" windowWidth="28800" windowHeight="17500" xr2:uid="{4E3EDB71-9423-764F-AB16-D8E153A84166}"/>
+    <workbookView xWindow="20" yWindow="620" windowWidth="51200" windowHeight="28180" activeTab="1" xr2:uid="{4E3EDB71-9423-764F-AB16-D8E153A84166}"/>
   </bookViews>
   <sheets>
     <sheet name="SWITCH_TO_SWITCH" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="77">
   <si>
     <t>Source</t>
   </si>
@@ -259,6 +259,15 @@
   </si>
   <si>
     <t>u19</t>
+  </si>
+  <si>
+    <t>fmn01</t>
+  </si>
+  <si>
+    <t>fmn02</t>
+  </si>
+  <si>
+    <t>u20</t>
   </si>
 </sst>
 </file>
@@ -385,10 +394,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -419,9 +427,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -459,7 +467,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -565,7 +573,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -707,7 +715,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -754,24 +762,22 @@
       </c>
     </row>
     <row r="15" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>31</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
         <v>21</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
+      <c r="O15">
         <v>32</v>
       </c>
-      <c r="P15" s="2" t="s">
+      <c r="P15" t="s">
         <v>32</v>
       </c>
-      <c r="Q15" s="2" t="s">
+      <c r="Q15" t="s">
         <v>19</v>
       </c>
       <c r="R15" t="s">
@@ -785,24 +791,22 @@
       </c>
     </row>
     <row r="16" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>31</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" t="s">
         <v>21</v>
       </c>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2">
+      <c r="O16">
         <v>31</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" t="s">
         <v>32</v>
       </c>
-      <c r="Q16" s="2" t="s">
+      <c r="Q16" t="s">
         <v>19</v>
       </c>
       <c r="R16" t="s">
@@ -816,24 +820,22 @@
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J17" s="2" t="s">
+      <c r="J17" t="s">
         <v>31</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L17" s="2" t="s">
+      <c r="K17" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2">
+      <c r="O17">
         <v>30</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="P17" t="s">
         <v>32</v>
       </c>
-      <c r="Q17" s="2" t="s">
+      <c r="Q17" t="s">
         <v>19</v>
       </c>
       <c r="R17" t="s">
@@ -847,24 +849,22 @@
       </c>
     </row>
     <row r="18" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J18" s="2" t="s">
+      <c r="J18" t="s">
         <v>31</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="K18" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" t="s">
         <v>21</v>
       </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18" t="s">
         <v>33</v>
       </c>
-      <c r="Q18" s="2" t="s">
+      <c r="Q18" t="s">
         <v>18</v>
       </c>
       <c r="R18" t="s">
@@ -875,24 +875,22 @@
       </c>
     </row>
     <row r="19" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J19" s="2" t="s">
+      <c r="J19" t="s">
         <v>31</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="K19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L19" t="s">
         <v>21</v>
       </c>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2">
-        <v>2</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="O19">
+        <v>2</v>
+      </c>
+      <c r="P19" t="s">
         <v>34</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="Q19" t="s">
         <v>18</v>
       </c>
       <c r="R19" t="s">
@@ -903,24 +901,22 @@
       </c>
     </row>
     <row r="20" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J20" s="2" t="s">
+      <c r="J20" t="s">
         <v>32</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="K20" t="s">
+        <v>19</v>
+      </c>
+      <c r="L20" t="s">
         <v>21</v>
       </c>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2">
-        <v>1</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20" t="s">
         <v>33</v>
       </c>
-      <c r="Q20" s="2" t="s">
+      <c r="Q20" t="s">
         <v>18</v>
       </c>
       <c r="R20" t="s">
@@ -931,24 +927,22 @@
       </c>
     </row>
     <row r="21" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J21" s="2" t="s">
+      <c r="J21" t="s">
         <v>32</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="K21" t="s">
+        <v>19</v>
+      </c>
+      <c r="L21" t="s">
         <v>21</v>
       </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2">
-        <v>2</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="O21">
+        <v>2</v>
+      </c>
+      <c r="P21" t="s">
         <v>34</v>
       </c>
-      <c r="Q21" s="2" t="s">
+      <c r="Q21" t="s">
         <v>18</v>
       </c>
       <c r="R21" t="s">
@@ -959,24 +953,22 @@
       </c>
     </row>
     <row r="22" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J22" s="2" t="s">
+      <c r="J22" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="K22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" t="s">
         <v>21</v>
       </c>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2">
+      <c r="O22">
         <v>3</v>
       </c>
-      <c r="P22" s="2" t="s">
+      <c r="P22" t="s">
         <v>35</v>
       </c>
-      <c r="Q22" s="2" t="s">
+      <c r="Q22" t="s">
         <v>19</v>
       </c>
       <c r="R22" t="s">
@@ -987,24 +979,22 @@
       </c>
     </row>
     <row r="23" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J23" s="2" t="s">
+      <c r="J23" t="s">
         <v>31</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="K23" t="s">
+        <v>18</v>
+      </c>
+      <c r="L23" t="s">
         <v>21</v>
       </c>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2">
+      <c r="O23">
         <v>4</v>
       </c>
-      <c r="P23" s="2" t="s">
+      <c r="P23" t="s">
         <v>36</v>
       </c>
-      <c r="Q23" s="2" t="s">
+      <c r="Q23" t="s">
         <v>19</v>
       </c>
       <c r="R23" t="s">
@@ -1015,24 +1005,22 @@
       </c>
     </row>
     <row r="24" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>32</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="L24" t="s">
         <v>21</v>
       </c>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2">
+      <c r="O24">
         <v>3</v>
       </c>
-      <c r="P24" s="2" t="s">
+      <c r="P24" t="s">
         <v>35</v>
       </c>
-      <c r="Q24" s="2" t="s">
+      <c r="Q24" t="s">
         <v>19</v>
       </c>
       <c r="R24" t="s">
@@ -1043,24 +1031,22 @@
       </c>
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>32</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L25" s="2" t="s">
+      <c r="K25" t="s">
+        <v>19</v>
+      </c>
+      <c r="L25" t="s">
         <v>21</v>
       </c>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2">
+      <c r="O25">
         <v>4</v>
       </c>
-      <c r="P25" s="2" t="s">
+      <c r="P25" t="s">
         <v>36</v>
       </c>
-      <c r="Q25" s="2" t="s">
+      <c r="Q25" t="s">
         <v>19</v>
       </c>
       <c r="R25" t="s">
@@ -1071,24 +1057,22 @@
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>33</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2">
+      <c r="K26" t="s">
+        <v>18</v>
+      </c>
+      <c r="L26" t="s">
+        <v>22</v>
+      </c>
+      <c r="O26">
         <v>56</v>
       </c>
-      <c r="P26" s="2" t="s">
+      <c r="P26" t="s">
         <v>34</v>
       </c>
-      <c r="Q26" s="2" t="s">
+      <c r="Q26" t="s">
         <v>18</v>
       </c>
       <c r="R26" t="s">
@@ -1102,24 +1086,22 @@
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>33</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2">
+      <c r="K27" t="s">
+        <v>18</v>
+      </c>
+      <c r="L27" t="s">
+        <v>22</v>
+      </c>
+      <c r="O27">
         <v>55</v>
       </c>
-      <c r="P27" s="2" t="s">
+      <c r="P27" t="s">
         <v>34</v>
       </c>
-      <c r="Q27" s="2" t="s">
+      <c r="Q27" t="s">
         <v>18</v>
       </c>
       <c r="R27" t="s">
@@ -1133,24 +1115,22 @@
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J28" s="2" t="s">
+      <c r="J28" t="s">
         <v>33</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2">
+      <c r="K28" t="s">
+        <v>18</v>
+      </c>
+      <c r="L28" t="s">
+        <v>22</v>
+      </c>
+      <c r="O28">
         <v>54</v>
       </c>
-      <c r="P28" s="2" t="s">
+      <c r="P28" t="s">
         <v>34</v>
       </c>
-      <c r="Q28" s="2" t="s">
+      <c r="Q28" t="s">
         <v>18</v>
       </c>
       <c r="R28" t="s">
@@ -1164,529 +1144,520 @@
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J29" s="2" t="s">
+      <c r="J29" t="s">
         <v>35</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2">
+      <c r="K29" t="s">
+        <v>19</v>
+      </c>
+      <c r="L29" t="s">
+        <v>22</v>
+      </c>
+      <c r="O29">
         <v>56</v>
       </c>
-      <c r="P29" s="2" t="s">
+      <c r="P29" t="s">
         <v>36</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R29" s="2" t="s">
+      <c r="Q29" t="s">
+        <v>19</v>
+      </c>
+      <c r="R29" t="s">
         <v>23</v>
       </c>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2">
+      <c r="T29">
         <v>56</v>
       </c>
-      <c r="U29" s="2" t="s">
+      <c r="U29" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J30" s="2" t="s">
+      <c r="J30" t="s">
         <v>35</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2">
+      <c r="K30" t="s">
+        <v>19</v>
+      </c>
+      <c r="L30" t="s">
+        <v>22</v>
+      </c>
+      <c r="O30">
         <v>55</v>
       </c>
-      <c r="P30" s="2" t="s">
+      <c r="P30" t="s">
         <v>36</v>
       </c>
-      <c r="Q30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R30" s="2" t="s">
+      <c r="Q30" t="s">
+        <v>19</v>
+      </c>
+      <c r="R30" t="s">
         <v>23</v>
       </c>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2">
+      <c r="T30">
         <v>55</v>
       </c>
-      <c r="U30" s="2" t="s">
+      <c r="U30" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J31" s="2" t="s">
+      <c r="J31" t="s">
         <v>35</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2">
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" t="s">
+        <v>22</v>
+      </c>
+      <c r="O31">
         <v>54</v>
       </c>
-      <c r="P31" s="2" t="s">
+      <c r="P31" t="s">
         <v>36</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R31" s="2" t="s">
+      <c r="Q31" t="s">
+        <v>19</v>
+      </c>
+      <c r="R31" t="s">
         <v>23</v>
       </c>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2">
+      <c r="T31">
         <v>54</v>
       </c>
-      <c r="U31" s="2" t="s">
+      <c r="U31" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J32" s="2" t="s">
+      <c r="J32" t="s">
         <v>39</v>
       </c>
-      <c r="K32" s="2" t="s">
+      <c r="K32" t="s">
         <v>20</v>
       </c>
-      <c r="L32" s="2" t="s">
+      <c r="L32" t="s">
         <v>21</v>
       </c>
-      <c r="O32" s="2">
+      <c r="O32">
         <v>52</v>
       </c>
-      <c r="P32" s="2" t="s">
+      <c r="P32" t="s">
         <v>40</v>
       </c>
-      <c r="Q32" s="2" t="s">
+      <c r="Q32" t="s">
         <v>20</v>
       </c>
-      <c r="R32" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T32" s="2">
+      <c r="R32" t="s">
+        <v>22</v>
+      </c>
+      <c r="T32">
         <v>52</v>
       </c>
-      <c r="U32" s="2" t="s">
+      <c r="U32" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J33" s="2" t="s">
+      <c r="J33" t="s">
         <v>39</v>
       </c>
-      <c r="K33" s="2" t="s">
+      <c r="K33" t="s">
         <v>20</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="L33" t="s">
         <v>21</v>
       </c>
-      <c r="O33" s="2">
+      <c r="O33">
         <v>51</v>
       </c>
-      <c r="P33" s="2" t="s">
+      <c r="P33" t="s">
         <v>40</v>
       </c>
-      <c r="Q33" s="2" t="s">
+      <c r="Q33" t="s">
         <v>20</v>
       </c>
-      <c r="R33" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T33" s="2">
+      <c r="R33" t="s">
+        <v>22</v>
+      </c>
+      <c r="T33">
         <v>51</v>
       </c>
-      <c r="U33" s="2" t="s">
+      <c r="U33" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="34" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J34" s="2" t="s">
+      <c r="J34" t="s">
         <v>39</v>
       </c>
-      <c r="K34" s="2" t="s">
+      <c r="K34" t="s">
         <v>20</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L34" t="s">
         <v>21</v>
       </c>
-      <c r="O34" s="2">
+      <c r="O34">
         <v>48</v>
       </c>
-      <c r="P34" s="2" t="s">
+      <c r="P34" t="s">
         <v>40</v>
       </c>
-      <c r="Q34" s="2" t="s">
+      <c r="Q34" t="s">
         <v>20</v>
       </c>
-      <c r="R34" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T34" s="2">
+      <c r="R34" t="s">
+        <v>22</v>
+      </c>
+      <c r="T34">
         <v>48</v>
       </c>
-      <c r="U34" s="2" t="s">
+      <c r="U34" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="35" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J35" s="2" t="s">
+      <c r="J35" t="s">
         <v>39</v>
       </c>
-      <c r="K35" s="2" t="s">
+      <c r="K35" t="s">
         <v>20</v>
       </c>
-      <c r="L35" s="2" t="s">
+      <c r="L35" t="s">
         <v>21</v>
       </c>
-      <c r="O35" s="2">
+      <c r="O35">
         <v>50</v>
       </c>
-      <c r="P35" s="2" t="s">
+      <c r="P35" t="s">
         <v>31</v>
       </c>
-      <c r="Q35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R35" s="2" t="s">
+      <c r="Q35" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" t="s">
         <v>21</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35">
         <v>5</v>
       </c>
     </row>
     <row r="36" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J36" s="2" t="s">
+      <c r="J36" t="s">
         <v>39</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K36" t="s">
         <v>20</v>
       </c>
-      <c r="L36" s="2" t="s">
+      <c r="L36" t="s">
         <v>21</v>
       </c>
-      <c r="O36" s="2">
+      <c r="O36">
         <v>49</v>
       </c>
-      <c r="P36" s="2" t="s">
+      <c r="P36" t="s">
         <v>32</v>
       </c>
-      <c r="Q36" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R36" s="2" t="s">
+      <c r="Q36" t="s">
+        <v>19</v>
+      </c>
+      <c r="R36" t="s">
         <v>21</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36">
         <v>5</v>
       </c>
     </row>
     <row r="37" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J37" s="2" t="s">
+      <c r="J37" t="s">
         <v>40</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="K37" t="s">
         <v>20</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O37" s="2">
+      <c r="L37" t="s">
+        <v>22</v>
+      </c>
+      <c r="O37">
         <v>50</v>
       </c>
-      <c r="P37" s="2" t="s">
+      <c r="P37" t="s">
         <v>31</v>
       </c>
-      <c r="Q37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R37" s="2" t="s">
+      <c r="Q37" t="s">
+        <v>18</v>
+      </c>
+      <c r="R37" t="s">
         <v>21</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37">
         <v>6</v>
       </c>
     </row>
     <row r="38" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J38" s="2" t="s">
+      <c r="J38" t="s">
         <v>40</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="K38" t="s">
         <v>20</v>
       </c>
-      <c r="L38" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O38" s="2">
+      <c r="L38" t="s">
+        <v>22</v>
+      </c>
+      <c r="O38">
         <v>49</v>
       </c>
-      <c r="P38" s="2" t="s">
+      <c r="P38" t="s">
         <v>32</v>
       </c>
-      <c r="Q38" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R38" s="2" t="s">
+      <c r="Q38" t="s">
+        <v>19</v>
+      </c>
+      <c r="R38" t="s">
         <v>21</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38">
         <v>6</v>
       </c>
     </row>
     <row r="39" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J39" s="2" t="s">
+      <c r="J39" t="s">
         <v>49</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="K39" t="s">
         <v>48</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="L39" t="s">
         <v>21</v>
       </c>
-      <c r="O39" s="2">
-        <v>1</v>
-      </c>
-      <c r="P39" s="2" t="s">
+      <c r="O39">
+        <v>1</v>
+      </c>
+      <c r="P39" t="s">
         <v>31</v>
       </c>
-      <c r="Q39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R39" s="2" t="s">
+      <c r="Q39" t="s">
+        <v>18</v>
+      </c>
+      <c r="R39" t="s">
         <v>21</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39">
         <v>7</v>
       </c>
     </row>
     <row r="40" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J40" s="2" t="s">
+      <c r="J40" t="s">
         <v>50</v>
       </c>
-      <c r="K40" s="2" t="s">
+      <c r="K40" t="s">
         <v>48</v>
       </c>
-      <c r="L40" s="2" t="s">
+      <c r="L40" t="s">
         <v>21</v>
       </c>
-      <c r="O40" s="2">
-        <v>1</v>
-      </c>
-      <c r="P40" s="2" t="s">
+      <c r="O40">
+        <v>1</v>
+      </c>
+      <c r="P40" t="s">
         <v>31</v>
       </c>
-      <c r="Q40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R40" s="2" t="s">
+      <c r="Q40" t="s">
+        <v>18</v>
+      </c>
+      <c r="R40" t="s">
         <v>21</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40">
         <v>8</v>
       </c>
     </row>
     <row r="41" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J41" s="2" t="s">
+      <c r="J41" t="s">
         <v>49</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="K41" t="s">
         <v>48</v>
       </c>
-      <c r="L41" s="2" t="s">
+      <c r="L41" t="s">
         <v>21</v>
       </c>
-      <c r="O41" s="2">
-        <v>2</v>
-      </c>
-      <c r="P41" s="2" t="s">
+      <c r="O41">
+        <v>2</v>
+      </c>
+      <c r="P41" t="s">
         <v>32</v>
       </c>
-      <c r="Q41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R41" s="2" t="s">
+      <c r="Q41" t="s">
+        <v>19</v>
+      </c>
+      <c r="R41" t="s">
         <v>21</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41">
         <v>7</v>
       </c>
     </row>
     <row r="42" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J42" s="2" t="s">
+      <c r="J42" t="s">
         <v>50</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="K42" t="s">
         <v>48</v>
       </c>
-      <c r="L42" s="2" t="s">
+      <c r="L42" t="s">
         <v>21</v>
       </c>
-      <c r="O42" s="2">
-        <v>2</v>
-      </c>
-      <c r="P42" s="2" t="s">
+      <c r="O42">
+        <v>2</v>
+      </c>
+      <c r="P42" t="s">
         <v>32</v>
       </c>
-      <c r="Q42" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R42" s="2" t="s">
+      <c r="Q42" t="s">
+        <v>19</v>
+      </c>
+      <c r="R42" t="s">
         <v>21</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42">
         <v>8</v>
       </c>
     </row>
     <row r="43" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J43" s="2" t="s">
+      <c r="J43" t="s">
         <v>38</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L43" s="2" t="s">
+      <c r="K43" t="s">
+        <v>18</v>
+      </c>
+      <c r="L43" t="s">
         <v>47</v>
       </c>
-      <c r="O43" s="2">
+      <c r="O43">
         <v>48</v>
       </c>
-      <c r="P43" s="2" t="s">
+      <c r="P43" t="s">
         <v>33</v>
       </c>
-      <c r="Q43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R43" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T43" s="2">
+      <c r="Q43" t="s">
+        <v>18</v>
+      </c>
+      <c r="R43" t="s">
+        <v>22</v>
+      </c>
+      <c r="T43">
         <v>51</v>
       </c>
     </row>
     <row r="44" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J44" s="2" t="s">
+      <c r="J44" t="s">
         <v>38</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L44" s="2" t="s">
+      <c r="K44" t="s">
+        <v>18</v>
+      </c>
+      <c r="L44" t="s">
         <v>47</v>
       </c>
-      <c r="O44" s="2">
+      <c r="O44">
         <v>47</v>
       </c>
-      <c r="P44" s="2" t="s">
+      <c r="P44" t="s">
         <v>34</v>
       </c>
-      <c r="Q44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R44" s="2" t="s">
+      <c r="Q44" t="s">
+        <v>18</v>
+      </c>
+      <c r="R44" t="s">
         <v>23</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44">
         <v>51</v>
       </c>
     </row>
     <row r="45" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J45" s="3" t="s">
+      <c r="J45" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K45" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L45" s="5" t="s">
+      <c r="K45" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="L45" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="N45" s="6" t="s">
+      <c r="N45" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O45" s="7">
-        <v>1</v>
-      </c>
-      <c r="P45" s="3" t="s">
+      <c r="O45" s="6">
+        <v>1</v>
+      </c>
+      <c r="P45" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Q45" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R45" s="5" t="s">
+      <c r="Q45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R45" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="T45" s="7">
+      <c r="T45" s="6">
         <v>29</v>
       </c>
     </row>
     <row r="46" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J46" s="3" t="s">
+      <c r="J46" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K46" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L46" s="5" t="s">
+      <c r="K46" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="L46" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="N46" s="6" t="s">
+      <c r="N46" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O46" s="7">
-        <v>2</v>
-      </c>
-      <c r="P46" s="3" t="s">
+      <c r="O46" s="6">
+        <v>2</v>
+      </c>
+      <c r="P46" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q46" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R46" s="5" t="s">
+      <c r="Q46" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R46" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T46" s="7">
+      <c r="T46" s="6">
         <v>29</v>
       </c>
     </row>
     <row r="47" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J47" s="3" t="s">
+      <c r="J47" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K47" s="4" t="s">
+      <c r="K47" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L47" t="s">
         <v>73</v>
       </c>
-      <c r="N47" s="6" t="s">
+      <c r="N47" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O47">
         <v>1</v>
       </c>
-      <c r="P47" s="3" t="s">
+      <c r="P47" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Q47" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R47" s="5" t="s">
+      <c r="Q47" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R47" s="4" t="s">
         <v>47</v>
       </c>
       <c r="T47">
@@ -1694,28 +1665,28 @@
       </c>
     </row>
     <row r="48" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J48" s="3" t="s">
+      <c r="J48" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K48" s="4" t="s">
+      <c r="K48" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L48" t="s">
         <v>73</v>
       </c>
-      <c r="N48" s="6" t="s">
+      <c r="N48" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O48">
         <v>2</v>
       </c>
-      <c r="P48" s="3" t="s">
+      <c r="P48" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q48" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R48" s="5" t="s">
+      <c r="Q48" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R48" s="4" t="s">
         <v>23</v>
       </c>
       <c r="T48">
@@ -1729,7 +1700,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6C3018C-CE0C-E04E-8947-8C874399EC7B}">
-  <dimension ref="J14:T53"/>
+  <dimension ref="J14:T57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -1770,1202 +1741,1250 @@
       </c>
     </row>
     <row r="15" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="M15" t="s">
         <v>16</v>
       </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
         <v>33</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2">
+      <c r="Q15" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" t="s">
+        <v>22</v>
+      </c>
+      <c r="T15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>6</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" t="s">
         <v>24</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M16" t="s">
         <v>16</v>
       </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2">
-        <v>2</v>
-      </c>
-      <c r="P16" s="2" t="s">
+      <c r="O16">
+        <v>2</v>
+      </c>
+      <c r="P16" t="s">
         <v>51</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2">
+      <c r="Q16" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" t="s">
+        <v>22</v>
+      </c>
+      <c r="T16">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J17" s="2" t="s">
+      <c r="J17" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L17" s="2" t="s">
+      <c r="K17" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" t="s">
         <v>24</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M17" t="s">
         <v>17</v>
       </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="s">
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17" t="s">
         <v>34</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R17" s="2" t="s">
+      <c r="Q17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R17" t="s">
         <v>23</v>
       </c>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2">
+      <c r="T17">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J18" s="2" t="s">
+      <c r="J18" t="s">
         <v>6</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="K18" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" t="s">
         <v>24</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M18" t="s">
         <v>17</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2">
-        <v>2</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="O18">
+        <v>2</v>
+      </c>
+      <c r="P18" t="s">
         <v>51</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R18" s="2" t="s">
+      <c r="Q18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R18" t="s">
         <v>23</v>
       </c>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2">
+      <c r="T18">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J19" s="2" t="s">
+      <c r="J19" t="s">
         <v>7</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="K19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L19" t="s">
         <v>25</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" t="s">
         <v>16</v>
       </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2">
-        <v>1</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19" t="s">
         <v>33</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R19" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2">
+      <c r="Q19" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" t="s">
+        <v>22</v>
+      </c>
+      <c r="T19">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J20" s="2" t="s">
+      <c r="J20" t="s">
         <v>7</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="K20" t="s">
+        <v>18</v>
+      </c>
+      <c r="L20" t="s">
         <v>25</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="M20" t="s">
         <v>16</v>
       </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2">
-        <v>2</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20">
+        <v>2</v>
+      </c>
+      <c r="P20" t="s">
         <v>51</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2">
+      <c r="Q20" t="s">
+        <v>18</v>
+      </c>
+      <c r="R20" t="s">
+        <v>22</v>
+      </c>
+      <c r="T20">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J21" s="2" t="s">
+      <c r="J21" t="s">
         <v>7</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="K21" t="s">
+        <v>18</v>
+      </c>
+      <c r="L21" t="s">
         <v>25</v>
       </c>
-      <c r="M21" s="2" t="s">
+      <c r="M21" t="s">
         <v>17</v>
       </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21" t="s">
         <v>34</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R21" s="2" t="s">
+      <c r="Q21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R21" t="s">
         <v>23</v>
       </c>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2">
+      <c r="T21">
         <v>3</v>
       </c>
     </row>
     <row r="22" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J22" s="2" t="s">
+      <c r="J22" t="s">
         <v>7</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="K22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" t="s">
         <v>25</v>
       </c>
-      <c r="M22" s="2" t="s">
+      <c r="M22" t="s">
         <v>17</v>
       </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2">
-        <v>2</v>
-      </c>
-      <c r="P22" s="2" t="s">
+      <c r="O22">
+        <v>2</v>
+      </c>
+      <c r="P22" t="s">
         <v>51</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="Q22" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" t="s">
         <v>23</v>
       </c>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2">
+      <c r="T22">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J23" s="2" t="s">
+      <c r="J23" t="s">
         <v>8</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="K23" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" t="s">
         <v>24</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="M23" t="s">
         <v>16</v>
       </c>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2">
-        <v>1</v>
-      </c>
-      <c r="P23" s="2" t="s">
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23" t="s">
         <v>35</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2">
+      <c r="Q23" t="s">
+        <v>19</v>
+      </c>
+      <c r="R23" t="s">
+        <v>22</v>
+      </c>
+      <c r="T23">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>8</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="L24" t="s">
         <v>24</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" t="s">
         <v>16</v>
       </c>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2">
-        <v>2</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="O24">
+        <v>2</v>
+      </c>
+      <c r="P24" t="s">
         <v>51</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2">
+      <c r="Q24" t="s">
+        <v>19</v>
+      </c>
+      <c r="R24" t="s">
+        <v>22</v>
+      </c>
+      <c r="T24">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>8</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L25" s="2" t="s">
+      <c r="K25" t="s">
+        <v>19</v>
+      </c>
+      <c r="L25" t="s">
         <v>24</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" t="s">
         <v>17</v>
       </c>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
         <v>36</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R25" s="2" t="s">
+      <c r="Q25" t="s">
+        <v>19</v>
+      </c>
+      <c r="R25" t="s">
         <v>23</v>
       </c>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2">
+      <c r="T25">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>8</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L26" s="2" t="s">
+      <c r="K26" t="s">
+        <v>19</v>
+      </c>
+      <c r="L26" t="s">
         <v>24</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" t="s">
         <v>17</v>
       </c>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2">
-        <v>2</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26">
+        <v>2</v>
+      </c>
+      <c r="P26" t="s">
         <v>51</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R26" s="2" t="s">
+      <c r="Q26" t="s">
+        <v>19</v>
+      </c>
+      <c r="R26" t="s">
         <v>23</v>
       </c>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2">
+      <c r="T26">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>9</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L27" s="2" t="s">
+      <c r="K27" t="s">
+        <v>18</v>
+      </c>
+      <c r="L27" t="s">
         <v>26</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" t="s">
         <v>16</v>
       </c>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
         <v>33</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R27" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2">
+      <c r="Q27" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" t="s">
+        <v>22</v>
+      </c>
+      <c r="T27">
         <v>5</v>
       </c>
     </row>
     <row r="28" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J28" s="2" t="s">
+      <c r="J28" t="s">
         <v>9</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L28" s="2" t="s">
+      <c r="K28" t="s">
+        <v>18</v>
+      </c>
+      <c r="L28" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" t="s">
         <v>16</v>
       </c>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2">
-        <v>2</v>
-      </c>
-      <c r="P28" s="2" t="s">
+      <c r="O28">
+        <v>2</v>
+      </c>
+      <c r="P28" t="s">
         <v>34</v>
       </c>
-      <c r="Q28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R28" s="2" t="s">
+      <c r="Q28" t="s">
+        <v>18</v>
+      </c>
+      <c r="R28" t="s">
         <v>23</v>
       </c>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2">
+      <c r="T28">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J29" s="2" t="s">
+      <c r="J29" t="s">
         <v>10</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L29" s="2" t="s">
+      <c r="K29" t="s">
+        <v>19</v>
+      </c>
+      <c r="L29" t="s">
         <v>25</v>
       </c>
-      <c r="M29" s="2" t="s">
+      <c r="M29" t="s">
         <v>16</v>
       </c>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2">
-        <v>1</v>
-      </c>
-      <c r="P29" s="2" t="s">
+      <c r="O29">
+        <v>1</v>
+      </c>
+      <c r="P29" t="s">
         <v>35</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2">
+      <c r="Q29" t="s">
+        <v>19</v>
+      </c>
+      <c r="R29" t="s">
+        <v>22</v>
+      </c>
+      <c r="T29">
         <v>3</v>
       </c>
     </row>
     <row r="30" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J30" s="2" t="s">
+      <c r="J30" t="s">
         <v>10</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L30" s="2" t="s">
+      <c r="K30" t="s">
+        <v>19</v>
+      </c>
+      <c r="L30" t="s">
         <v>25</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="M30" t="s">
         <v>16</v>
       </c>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2">
-        <v>2</v>
-      </c>
-      <c r="P30" s="2" t="s">
+      <c r="O30">
+        <v>2</v>
+      </c>
+      <c r="P30" t="s">
         <v>36</v>
       </c>
-      <c r="Q30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R30" s="2" t="s">
+      <c r="Q30" t="s">
+        <v>19</v>
+      </c>
+      <c r="R30" t="s">
         <v>23</v>
       </c>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2">
+      <c r="T30">
         <v>3</v>
       </c>
     </row>
     <row r="31" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J31" s="2" t="s">
+      <c r="J31" t="s">
         <v>11</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L31" s="2" t="s">
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" t="s">
         <v>26</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="M31" t="s">
         <v>16</v>
       </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2">
-        <v>1</v>
-      </c>
-      <c r="P31" s="2" t="s">
+      <c r="O31">
+        <v>1</v>
+      </c>
+      <c r="P31" t="s">
         <v>35</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2">
+      <c r="Q31" t="s">
+        <v>19</v>
+      </c>
+      <c r="R31" t="s">
+        <v>22</v>
+      </c>
+      <c r="T31">
         <v>4</v>
       </c>
     </row>
     <row r="32" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J32" s="2" t="s">
+      <c r="J32" t="s">
         <v>11</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L32" s="2" t="s">
+      <c r="K32" t="s">
+        <v>19</v>
+      </c>
+      <c r="L32" t="s">
         <v>26</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" t="s">
         <v>16</v>
       </c>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2">
-        <v>2</v>
-      </c>
-      <c r="P32" s="2" t="s">
+      <c r="O32">
+        <v>2</v>
+      </c>
+      <c r="P32" t="s">
         <v>36</v>
       </c>
-      <c r="Q32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R32" s="2" t="s">
+      <c r="Q32" t="s">
+        <v>19</v>
+      </c>
+      <c r="R32" t="s">
         <v>23</v>
       </c>
-      <c r="S32" s="2"/>
-      <c r="T32" s="2">
+      <c r="T32">
         <v>4</v>
       </c>
     </row>
     <row r="33" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J33" s="2" t="s">
+      <c r="J33" t="s">
         <v>12</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="K33" t="s">
+        <v>18</v>
+      </c>
+      <c r="L33" t="s">
         <v>27</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="M33" t="s">
         <v>16</v>
       </c>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="s">
+      <c r="O33">
+        <v>1</v>
+      </c>
+      <c r="P33" t="s">
         <v>33</v>
       </c>
-      <c r="Q33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S33" s="2"/>
-      <c r="T33" s="2">
+      <c r="Q33" t="s">
+        <v>18</v>
+      </c>
+      <c r="R33" t="s">
+        <v>22</v>
+      </c>
+      <c r="T33">
         <v>7</v>
       </c>
     </row>
     <row r="34" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J34" s="2" t="s">
+      <c r="J34" t="s">
         <v>12</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="K34" t="s">
+        <v>18</v>
+      </c>
+      <c r="L34" t="s">
         <v>27</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" t="s">
         <v>16</v>
       </c>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2">
-        <v>2</v>
-      </c>
-      <c r="P34" s="2" t="s">
+      <c r="O34">
+        <v>2</v>
+      </c>
+      <c r="P34" t="s">
         <v>33</v>
       </c>
-      <c r="Q34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R34" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S34" s="2"/>
-      <c r="T34" s="2">
+      <c r="Q34" t="s">
+        <v>18</v>
+      </c>
+      <c r="R34" t="s">
+        <v>22</v>
+      </c>
+      <c r="T34">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J35" s="2" t="s">
+      <c r="J35" t="s">
         <v>12</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L35" s="2" t="s">
+      <c r="K35" t="s">
+        <v>18</v>
+      </c>
+      <c r="L35" t="s">
         <v>27</v>
       </c>
-      <c r="M35" s="2" t="s">
+      <c r="M35" t="s">
         <v>17</v>
       </c>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2">
-        <v>1</v>
-      </c>
-      <c r="P35" s="2" t="s">
+      <c r="O35">
+        <v>1</v>
+      </c>
+      <c r="P35" t="s">
         <v>34</v>
       </c>
-      <c r="Q35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R35" s="2" t="s">
+      <c r="Q35" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" t="s">
         <v>23</v>
       </c>
-      <c r="S35" s="2"/>
-      <c r="T35" s="2">
+      <c r="T35">
         <v>7</v>
       </c>
     </row>
     <row r="36" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J36" s="2" t="s">
+      <c r="J36" t="s">
         <v>12</v>
       </c>
-      <c r="K36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L36" s="2" t="s">
+      <c r="K36" t="s">
+        <v>18</v>
+      </c>
+      <c r="L36" t="s">
         <v>27</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="M36" t="s">
         <v>17</v>
       </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2">
-        <v>2</v>
-      </c>
-      <c r="P36" s="2" t="s">
+      <c r="O36">
+        <v>2</v>
+      </c>
+      <c r="P36" t="s">
         <v>34</v>
       </c>
-      <c r="Q36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R36" s="2" t="s">
+      <c r="Q36" t="s">
+        <v>18</v>
+      </c>
+      <c r="R36" t="s">
         <v>23</v>
       </c>
-      <c r="S36" s="2"/>
-      <c r="T36" s="2">
+      <c r="T36">
         <v>8</v>
       </c>
     </row>
     <row r="37" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J37" s="2" t="s">
+      <c r="J37" t="s">
         <v>13</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L37" s="2" t="s">
+      <c r="K37" t="s">
+        <v>18</v>
+      </c>
+      <c r="L37" t="s">
         <v>28</v>
       </c>
-      <c r="M37" s="2" t="s">
+      <c r="M37" t="s">
         <v>16</v>
       </c>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2">
-        <v>1</v>
-      </c>
-      <c r="P37" s="2" t="s">
+      <c r="O37">
+        <v>1</v>
+      </c>
+      <c r="P37" t="s">
         <v>33</v>
       </c>
-      <c r="Q37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R37" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S37" s="2"/>
-      <c r="T37" s="2">
+      <c r="Q37" t="s">
+        <v>18</v>
+      </c>
+      <c r="R37" t="s">
+        <v>22</v>
+      </c>
+      <c r="T37">
         <v>9</v>
       </c>
     </row>
     <row r="38" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J38" s="2" t="s">
+      <c r="J38" t="s">
         <v>13</v>
       </c>
-      <c r="K38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L38" s="2" t="s">
+      <c r="K38" t="s">
+        <v>18</v>
+      </c>
+      <c r="L38" t="s">
         <v>28</v>
       </c>
-      <c r="M38" s="2" t="s">
+      <c r="M38" t="s">
         <v>16</v>
       </c>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2">
-        <v>2</v>
-      </c>
-      <c r="P38" s="2" t="s">
+      <c r="O38">
+        <v>2</v>
+      </c>
+      <c r="P38" t="s">
         <v>33</v>
       </c>
-      <c r="Q38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R38" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S38" s="2"/>
-      <c r="T38" s="2">
+      <c r="Q38" t="s">
+        <v>18</v>
+      </c>
+      <c r="R38" t="s">
+        <v>22</v>
+      </c>
+      <c r="T38">
         <v>10</v>
       </c>
     </row>
     <row r="39" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J39" s="2" t="s">
+      <c r="J39" t="s">
         <v>13</v>
       </c>
-      <c r="K39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L39" s="2" t="s">
+      <c r="K39" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" t="s">
         <v>28</v>
       </c>
-      <c r="M39" s="2" t="s">
+      <c r="M39" t="s">
         <v>17</v>
       </c>
-      <c r="N39" s="2"/>
-      <c r="O39" s="2">
-        <v>1</v>
-      </c>
-      <c r="P39" s="2" t="s">
+      <c r="O39">
+        <v>1</v>
+      </c>
+      <c r="P39" t="s">
         <v>34</v>
       </c>
-      <c r="Q39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R39" s="2" t="s">
+      <c r="Q39" t="s">
+        <v>18</v>
+      </c>
+      <c r="R39" t="s">
         <v>23</v>
       </c>
-      <c r="S39" s="2"/>
-      <c r="T39" s="2">
+      <c r="T39">
         <v>9</v>
       </c>
     </row>
     <row r="40" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J40" s="2" t="s">
+      <c r="J40" t="s">
         <v>13</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L40" s="2" t="s">
+      <c r="K40" t="s">
+        <v>18</v>
+      </c>
+      <c r="L40" t="s">
         <v>28</v>
       </c>
-      <c r="M40" s="2" t="s">
+      <c r="M40" t="s">
         <v>17</v>
       </c>
-      <c r="N40" s="2"/>
-      <c r="O40" s="2">
-        <v>2</v>
-      </c>
-      <c r="P40" s="2" t="s">
+      <c r="O40">
+        <v>2</v>
+      </c>
+      <c r="P40" t="s">
         <v>34</v>
       </c>
-      <c r="Q40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R40" s="2" t="s">
+      <c r="Q40" t="s">
+        <v>18</v>
+      </c>
+      <c r="R40" t="s">
         <v>23</v>
       </c>
-      <c r="S40" s="2"/>
-      <c r="T40" s="2">
+      <c r="T40">
         <v>10</v>
       </c>
     </row>
     <row r="41" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J41" s="2" t="s">
+      <c r="J41" t="s">
         <v>14</v>
       </c>
-      <c r="K41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L41" s="2" t="s">
+      <c r="K41" t="s">
+        <v>19</v>
+      </c>
+      <c r="L41" t="s">
         <v>27</v>
       </c>
-      <c r="M41" s="2" t="s">
+      <c r="M41" t="s">
         <v>16</v>
       </c>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2">
-        <v>1</v>
-      </c>
-      <c r="P41" s="2" t="s">
+      <c r="O41">
+        <v>1</v>
+      </c>
+      <c r="P41" t="s">
         <v>35</v>
       </c>
-      <c r="Q41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S41" s="2"/>
-      <c r="T41" s="2">
+      <c r="Q41" t="s">
+        <v>19</v>
+      </c>
+      <c r="R41" t="s">
+        <v>22</v>
+      </c>
+      <c r="T41">
         <v>5</v>
       </c>
     </row>
     <row r="42" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J42" s="2" t="s">
+      <c r="J42" t="s">
         <v>14</v>
       </c>
-      <c r="K42" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L42" s="2" t="s">
+      <c r="K42" t="s">
+        <v>19</v>
+      </c>
+      <c r="L42" t="s">
         <v>27</v>
       </c>
-      <c r="M42" s="2" t="s">
+      <c r="M42" t="s">
         <v>16</v>
       </c>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2">
-        <v>2</v>
-      </c>
-      <c r="P42" s="2" t="s">
+      <c r="O42">
+        <v>2</v>
+      </c>
+      <c r="P42" t="s">
         <v>35</v>
       </c>
-      <c r="Q42" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R42" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S42" s="2"/>
-      <c r="T42" s="2">
+      <c r="Q42" t="s">
+        <v>19</v>
+      </c>
+      <c r="R42" t="s">
+        <v>22</v>
+      </c>
+      <c r="T42">
         <v>6</v>
       </c>
     </row>
     <row r="43" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J43" s="2" t="s">
+      <c r="J43" t="s">
         <v>14</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L43" s="2" t="s">
+      <c r="K43" t="s">
+        <v>19</v>
+      </c>
+      <c r="L43" t="s">
         <v>27</v>
       </c>
-      <c r="M43" s="2" t="s">
+      <c r="M43" t="s">
         <v>17</v>
       </c>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2">
-        <v>1</v>
-      </c>
-      <c r="P43" s="2" t="s">
+      <c r="O43">
+        <v>1</v>
+      </c>
+      <c r="P43" t="s">
         <v>36</v>
       </c>
-      <c r="Q43" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R43" s="2" t="s">
+      <c r="Q43" t="s">
+        <v>19</v>
+      </c>
+      <c r="R43" t="s">
         <v>23</v>
       </c>
-      <c r="S43" s="2"/>
-      <c r="T43" s="2">
+      <c r="T43">
         <v>5</v>
       </c>
     </row>
     <row r="44" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J44" s="2" t="s">
+      <c r="J44" t="s">
         <v>14</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L44" s="2" t="s">
+      <c r="K44" t="s">
+        <v>19</v>
+      </c>
+      <c r="L44" t="s">
         <v>27</v>
       </c>
-      <c r="M44" s="2" t="s">
+      <c r="M44" t="s">
         <v>17</v>
       </c>
-      <c r="N44" s="2"/>
-      <c r="O44" s="2">
-        <v>2</v>
-      </c>
-      <c r="P44" s="2" t="s">
+      <c r="O44">
+        <v>2</v>
+      </c>
+      <c r="P44" t="s">
         <v>36</v>
       </c>
-      <c r="Q44" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R44" s="2" t="s">
+      <c r="Q44" t="s">
+        <v>19</v>
+      </c>
+      <c r="R44" t="s">
         <v>23</v>
       </c>
-      <c r="S44" s="2"/>
-      <c r="T44" s="2">
+      <c r="T44">
         <v>6</v>
       </c>
     </row>
     <row r="45" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J45" s="2" t="s">
+      <c r="J45" t="s">
         <v>15</v>
       </c>
-      <c r="K45" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L45" s="2" t="s">
+      <c r="K45" t="s">
+        <v>19</v>
+      </c>
+      <c r="L45" t="s">
         <v>28</v>
       </c>
-      <c r="M45" s="2" t="s">
+      <c r="M45" t="s">
         <v>16</v>
       </c>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2">
-        <v>1</v>
-      </c>
-      <c r="P45" s="2" t="s">
+      <c r="O45">
+        <v>1</v>
+      </c>
+      <c r="P45" t="s">
         <v>35</v>
       </c>
-      <c r="Q45" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R45" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2">
+      <c r="Q45" t="s">
+        <v>19</v>
+      </c>
+      <c r="R45" t="s">
+        <v>22</v>
+      </c>
+      <c r="T45">
         <v>7</v>
       </c>
     </row>
     <row r="46" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J46" s="2" t="s">
+      <c r="J46" t="s">
         <v>15</v>
       </c>
-      <c r="K46" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L46" s="2" t="s">
+      <c r="K46" t="s">
+        <v>19</v>
+      </c>
+      <c r="L46" t="s">
         <v>28</v>
       </c>
-      <c r="M46" s="2" t="s">
+      <c r="M46" t="s">
         <v>16</v>
       </c>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2">
-        <v>2</v>
-      </c>
-      <c r="P46" s="2" t="s">
+      <c r="O46">
+        <v>2</v>
+      </c>
+      <c r="P46" t="s">
         <v>35</v>
       </c>
-      <c r="Q46" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R46" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S46" s="2"/>
-      <c r="T46" s="2">
+      <c r="Q46" t="s">
+        <v>19</v>
+      </c>
+      <c r="R46" t="s">
+        <v>22</v>
+      </c>
+      <c r="T46">
         <v>8</v>
       </c>
     </row>
     <row r="47" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J47" s="2" t="s">
+      <c r="J47" t="s">
         <v>15</v>
       </c>
-      <c r="K47" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L47" s="2" t="s">
+      <c r="K47" t="s">
+        <v>19</v>
+      </c>
+      <c r="L47" t="s">
         <v>28</v>
       </c>
-      <c r="M47" s="2" t="s">
+      <c r="M47" t="s">
         <v>17</v>
       </c>
-      <c r="N47" s="2"/>
-      <c r="O47" s="2">
-        <v>1</v>
-      </c>
-      <c r="P47" s="2" t="s">
+      <c r="O47">
+        <v>1</v>
+      </c>
+      <c r="P47" t="s">
         <v>36</v>
       </c>
-      <c r="Q47" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R47" s="2" t="s">
+      <c r="Q47" t="s">
+        <v>19</v>
+      </c>
+      <c r="R47" t="s">
         <v>23</v>
       </c>
-      <c r="S47" s="2"/>
-      <c r="T47" s="2">
+      <c r="T47">
         <v>7</v>
       </c>
     </row>
     <row r="48" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J48" s="2" t="s">
+      <c r="J48" t="s">
         <v>15</v>
       </c>
-      <c r="K48" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L48" s="2" t="s">
+      <c r="K48" t="s">
+        <v>19</v>
+      </c>
+      <c r="L48" t="s">
         <v>28</v>
       </c>
-      <c r="M48" s="2" t="s">
+      <c r="M48" t="s">
         <v>17</v>
       </c>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2">
-        <v>2</v>
-      </c>
-      <c r="P48" s="2" t="s">
+      <c r="O48">
+        <v>2</v>
+      </c>
+      <c r="P48" t="s">
         <v>36</v>
       </c>
-      <c r="Q48" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R48" s="2" t="s">
+      <c r="Q48" t="s">
+        <v>19</v>
+      </c>
+      <c r="R48" t="s">
         <v>23</v>
       </c>
-      <c r="S48" s="2"/>
-      <c r="T48" s="2">
+      <c r="T48">
         <v>8</v>
       </c>
     </row>
     <row r="49" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J49" s="2" t="s">
+      <c r="J49" t="s">
         <v>67</v>
       </c>
-      <c r="K49" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L49" s="2" t="s">
+      <c r="K49" t="s">
+        <v>19</v>
+      </c>
+      <c r="L49" t="s">
         <v>68</v>
       </c>
-      <c r="M49" s="2" t="s">
+      <c r="M49" t="s">
         <v>16</v>
       </c>
-      <c r="O49" s="2">
-        <v>1</v>
-      </c>
-      <c r="P49" s="2" t="s">
+      <c r="O49">
+        <v>1</v>
+      </c>
+      <c r="P49" t="s">
         <v>35</v>
       </c>
-      <c r="Q49" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R49" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T49" s="2">
+      <c r="Q49" t="s">
+        <v>19</v>
+      </c>
+      <c r="R49" t="s">
+        <v>22</v>
+      </c>
+      <c r="T49">
         <v>9</v>
       </c>
     </row>
     <row r="50" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J50" s="2" t="s">
+      <c r="J50" t="s">
         <v>67</v>
       </c>
-      <c r="K50" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L50" s="2" t="s">
+      <c r="K50" t="s">
+        <v>19</v>
+      </c>
+      <c r="L50" t="s">
         <v>68</v>
       </c>
-      <c r="M50" s="2" t="s">
+      <c r="M50" t="s">
         <v>16</v>
       </c>
-      <c r="O50" s="2">
-        <v>2</v>
-      </c>
-      <c r="P50" s="2" t="s">
+      <c r="O50">
+        <v>2</v>
+      </c>
+      <c r="P50" t="s">
         <v>35</v>
       </c>
-      <c r="Q50" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R50" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T50" s="2">
+      <c r="Q50" t="s">
+        <v>19</v>
+      </c>
+      <c r="R50" t="s">
+        <v>22</v>
+      </c>
+      <c r="T50">
         <v>10</v>
       </c>
     </row>
     <row r="51" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J51" s="2" t="s">
+      <c r="J51" t="s">
         <v>67</v>
       </c>
-      <c r="K51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L51" s="2" t="s">
+      <c r="K51" t="s">
+        <v>19</v>
+      </c>
+      <c r="L51" t="s">
         <v>68</v>
       </c>
-      <c r="M51" s="2" t="s">
+      <c r="M51" t="s">
         <v>17</v>
       </c>
-      <c r="O51" s="2">
-        <v>1</v>
-      </c>
-      <c r="P51" s="2" t="s">
+      <c r="O51">
+        <v>1</v>
+      </c>
+      <c r="P51" t="s">
         <v>36</v>
       </c>
-      <c r="Q51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R51" s="2" t="s">
+      <c r="Q51" t="s">
+        <v>19</v>
+      </c>
+      <c r="R51" t="s">
         <v>23</v>
       </c>
-      <c r="T51" s="2">
+      <c r="T51">
         <v>9</v>
       </c>
     </row>
     <row r="52" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J52" s="2" t="s">
+      <c r="J52" t="s">
         <v>67</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L52" s="2" t="s">
+      <c r="K52" t="s">
+        <v>19</v>
+      </c>
+      <c r="L52" t="s">
         <v>68</v>
       </c>
-      <c r="M52" s="2" t="s">
+      <c r="M52" t="s">
         <v>17</v>
       </c>
-      <c r="O52" s="2">
-        <v>2</v>
-      </c>
-      <c r="P52" s="2" t="s">
+      <c r="O52">
+        <v>2</v>
+      </c>
+      <c r="P52" t="s">
         <v>36</v>
       </c>
-      <c r="Q52" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R52" s="2" t="s">
+      <c r="Q52" t="s">
+        <v>19</v>
+      </c>
+      <c r="R52" t="s">
         <v>23</v>
       </c>
-      <c r="T52" s="2">
+      <c r="T52">
         <v>10</v>
       </c>
     </row>
     <row r="53" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J53" s="2" t="s">
+      <c r="J53" t="s">
         <v>66</v>
       </c>
-      <c r="K53" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L53" s="2" t="s">
+      <c r="K53" t="s">
+        <v>19</v>
+      </c>
+      <c r="L53" t="s">
         <v>68</v>
       </c>
-      <c r="M53" s="2" t="s">
+      <c r="M53" t="s">
         <v>16</v>
       </c>
-      <c r="O53" s="2">
-        <v>1</v>
-      </c>
-      <c r="P53" s="2" t="s">
+      <c r="O53">
+        <v>1</v>
+      </c>
+      <c r="P53" t="s">
         <v>38</v>
       </c>
-      <c r="Q53" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R53" s="2" t="s">
+      <c r="Q53" t="s">
+        <v>18</v>
+      </c>
+      <c r="R53" t="s">
         <v>47</v>
       </c>
-      <c r="T53" s="2">
+      <c r="T53">
         <v>28</v>
+      </c>
+    </row>
+    <row r="54" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J54" t="s">
+        <v>74</v>
+      </c>
+      <c r="K54" t="s">
+        <v>18</v>
+      </c>
+      <c r="L54" t="s">
+        <v>76</v>
+      </c>
+      <c r="M54" t="s">
+        <v>16</v>
+      </c>
+      <c r="O54">
+        <v>1</v>
+      </c>
+      <c r="P54" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>18</v>
+      </c>
+      <c r="R54" t="s">
+        <v>22</v>
+      </c>
+      <c r="T54">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J55" t="s">
+        <v>74</v>
+      </c>
+      <c r="K55" t="s">
+        <v>18</v>
+      </c>
+      <c r="L55" t="s">
+        <v>76</v>
+      </c>
+      <c r="M55" t="s">
+        <v>16</v>
+      </c>
+      <c r="O55">
+        <v>2</v>
+      </c>
+      <c r="P55" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>18</v>
+      </c>
+      <c r="R55" t="s">
+        <v>23</v>
+      </c>
+      <c r="T55">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J56" t="s">
+        <v>75</v>
+      </c>
+      <c r="K56" t="s">
+        <v>19</v>
+      </c>
+      <c r="L56" t="s">
+        <v>76</v>
+      </c>
+      <c r="M56" t="s">
+        <v>16</v>
+      </c>
+      <c r="O56">
+        <v>1</v>
+      </c>
+      <c r="P56" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>19</v>
+      </c>
+      <c r="R56" t="s">
+        <v>22</v>
+      </c>
+      <c r="T56">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J57" t="s">
+        <v>75</v>
+      </c>
+      <c r="K57" t="s">
+        <v>19</v>
+      </c>
+      <c r="L57" t="s">
+        <v>76</v>
+      </c>
+      <c r="M57" t="s">
+        <v>16</v>
+      </c>
+      <c r="O57">
+        <v>2</v>
+      </c>
+      <c r="P57" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>19</v>
+      </c>
+      <c r="R57" t="s">
+        <v>23</v>
+      </c>
+      <c r="T57">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2975,7 +2994,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7990636-0CF9-6941-8EF6-80CF48D8BDA7}">
-  <dimension ref="J14:T34"/>
+  <dimension ref="J14:T36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="16" max="16" width="14.5" bestFit="1" customWidth="1"/>
@@ -3013,606 +3032,641 @@
       </c>
     </row>
     <row r="15" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="M15" t="s">
         <v>37</v>
       </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
         <v>38</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="2" t="s">
+      <c r="Q15" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" t="s">
         <v>47</v>
       </c>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2">
+      <c r="T15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>7</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" t="s">
         <v>25</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M16" t="s">
         <v>37</v>
       </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2">
-        <v>1</v>
-      </c>
-      <c r="P16" s="2" t="s">
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16" t="s">
         <v>38</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="2" t="s">
+      <c r="Q16" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" t="s">
         <v>47</v>
       </c>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2">
+      <c r="T16">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J17" s="2" t="s">
+      <c r="J17" t="s">
         <v>8</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L17" s="2" t="s">
+      <c r="K17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L17" t="s">
         <v>24</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M17" t="s">
         <v>37</v>
       </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="s">
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17" t="s">
         <v>38</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R17" s="2" t="s">
+      <c r="Q17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R17" t="s">
         <v>47</v>
       </c>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2">
+      <c r="T17">
         <v>3</v>
       </c>
     </row>
     <row r="18" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J18" s="2" t="s">
+      <c r="J18" t="s">
         <v>9</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="K18" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M18" t="s">
         <v>37</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R18" s="2" t="s">
+      <c r="Q18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R18" t="s">
         <v>47</v>
       </c>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2">
+      <c r="T18">
         <v>4</v>
       </c>
     </row>
     <row r="19" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J19" s="2" t="s">
+      <c r="J19" t="s">
         <v>10</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="K19" t="s">
+        <v>19</v>
+      </c>
+      <c r="L19" t="s">
         <v>25</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" t="s">
         <v>37</v>
       </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2">
-        <v>1</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19" t="s">
         <v>38</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R19" s="2" t="s">
+      <c r="Q19" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" t="s">
         <v>47</v>
       </c>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2">
+      <c r="T19">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J20" s="2" t="s">
+      <c r="J20" t="s">
         <v>11</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="K20" t="s">
+        <v>19</v>
+      </c>
+      <c r="L20" t="s">
         <v>26</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="M20" t="s">
         <v>37</v>
       </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2">
-        <v>1</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20" t="s">
         <v>38</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R20" s="2" t="s">
+      <c r="Q20" t="s">
+        <v>18</v>
+      </c>
+      <c r="R20" t="s">
         <v>47</v>
       </c>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2">
+      <c r="T20">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J21" s="2" t="s">
+      <c r="J21" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="K21" t="s">
+        <v>18</v>
+      </c>
+      <c r="L21" t="s">
         <v>27</v>
       </c>
-      <c r="M21" s="2" t="s">
+      <c r="M21" t="s">
         <v>37</v>
       </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21" t="s">
         <v>38</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R21" s="2" t="s">
+      <c r="Q21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R21" t="s">
         <v>47</v>
       </c>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2">
+      <c r="T21">
         <v>7</v>
       </c>
     </row>
     <row r="22" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J22" s="2" t="s">
+      <c r="J22" t="s">
         <v>13</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="K22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" t="s">
         <v>28</v>
       </c>
-      <c r="M22" s="2" t="s">
+      <c r="M22" t="s">
         <v>37</v>
       </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2">
-        <v>1</v>
-      </c>
-      <c r="P22" s="2" t="s">
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22" t="s">
         <v>38</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="Q22" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" t="s">
         <v>47</v>
       </c>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2">
+      <c r="T22">
         <v>8</v>
       </c>
     </row>
     <row r="23" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J23" s="2" t="s">
+      <c r="J23" t="s">
         <v>14</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="K23" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" t="s">
         <v>27</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="M23" t="s">
         <v>37</v>
       </c>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2">
-        <v>1</v>
-      </c>
-      <c r="P23" s="2" t="s">
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23" t="s">
         <v>38</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R23" s="2" t="s">
+      <c r="Q23" t="s">
+        <v>18</v>
+      </c>
+      <c r="R23" t="s">
         <v>47</v>
       </c>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2">
+      <c r="T23">
         <v>9</v>
       </c>
     </row>
     <row r="24" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>15</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="L24" t="s">
         <v>28</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" t="s">
         <v>37</v>
       </c>
-      <c r="O24" s="2">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24" t="s">
         <v>38</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R24" s="2" t="s">
+      <c r="Q24" t="s">
+        <v>18</v>
+      </c>
+      <c r="R24" t="s">
         <v>47</v>
       </c>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2">
+      <c r="T24">
         <v>10</v>
       </c>
     </row>
     <row r="25" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>52</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="K25" t="s">
         <v>20</v>
       </c>
-      <c r="L25" s="2" t="s">
+      <c r="L25" t="s">
         <v>56</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" t="s">
         <v>37</v>
       </c>
-      <c r="O25" s="2">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
         <v>38</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R25" s="2" t="s">
+      <c r="Q25" t="s">
+        <v>18</v>
+      </c>
+      <c r="R25" t="s">
         <v>47</v>
       </c>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2">
+      <c r="T25">
         <v>11</v>
       </c>
     </row>
     <row r="26" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>53</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K26" t="s">
         <v>20</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="L26" t="s">
         <v>57</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" t="s">
         <v>37</v>
       </c>
-      <c r="O26" s="2">
-        <v>1</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26">
+        <v>1</v>
+      </c>
+      <c r="P26" t="s">
         <v>38</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R26" s="2" t="s">
+      <c r="Q26" t="s">
+        <v>18</v>
+      </c>
+      <c r="R26" t="s">
         <v>47</v>
       </c>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2">
+      <c r="T26">
         <v>12</v>
       </c>
     </row>
     <row r="27" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>54</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K27" t="s">
         <v>20</v>
       </c>
-      <c r="L27" s="2" t="s">
+      <c r="L27" t="s">
         <v>58</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" t="s">
         <v>37</v>
       </c>
-      <c r="O27" s="2">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
         <v>38</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="Q27" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" t="s">
         <v>47</v>
       </c>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2">
+      <c r="T27">
         <v>13</v>
       </c>
     </row>
     <row r="28" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J28" s="2" t="s">
+      <c r="J28" t="s">
         <v>55</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="K28" t="s">
         <v>20</v>
       </c>
-      <c r="L28" s="2" t="s">
+      <c r="L28" t="s">
         <v>59</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" t="s">
         <v>37</v>
       </c>
-      <c r="O28" s="2">
-        <v>1</v>
-      </c>
-      <c r="P28" s="2" t="s">
+      <c r="O28">
+        <v>1</v>
+      </c>
+      <c r="P28" t="s">
         <v>38</v>
       </c>
-      <c r="Q28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R28" s="2" t="s">
+      <c r="Q28" t="s">
+        <v>18</v>
+      </c>
+      <c r="R28" t="s">
         <v>47</v>
       </c>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2">
+      <c r="T28">
         <v>14</v>
       </c>
     </row>
     <row r="29" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J29" s="2" t="s">
+      <c r="J29" t="s">
         <v>61</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L29" s="2" t="s">
+      <c r="K29" t="s">
+        <v>18</v>
+      </c>
+      <c r="L29" t="s">
         <v>62</v>
       </c>
-      <c r="M29" s="2" t="s">
+      <c r="M29" t="s">
         <v>37</v>
       </c>
-      <c r="O29" s="2">
-        <v>1</v>
-      </c>
-      <c r="P29" s="2" t="s">
+      <c r="O29">
+        <v>1</v>
+      </c>
+      <c r="P29" t="s">
         <v>38</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R29" s="2" t="s">
+      <c r="Q29" t="s">
+        <v>18</v>
+      </c>
+      <c r="R29" t="s">
         <v>47</v>
       </c>
-      <c r="T29" s="2">
+      <c r="T29">
         <v>15</v>
       </c>
     </row>
     <row r="30" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J30" s="2" t="s">
+      <c r="J30" t="s">
         <v>63</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L30" s="2" t="s">
+      <c r="K30" t="s">
+        <v>18</v>
+      </c>
+      <c r="L30" t="s">
         <v>62</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="M30" t="s">
         <v>37</v>
       </c>
-      <c r="O30" s="2">
-        <v>1</v>
-      </c>
-      <c r="P30" s="2" t="s">
+      <c r="O30">
+        <v>1</v>
+      </c>
+      <c r="P30" t="s">
         <v>38</v>
       </c>
-      <c r="Q30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R30" s="2" t="s">
+      <c r="Q30" t="s">
+        <v>18</v>
+      </c>
+      <c r="R30" t="s">
         <v>47</v>
       </c>
-      <c r="T30" s="2">
+      <c r="T30">
         <v>16</v>
       </c>
     </row>
     <row r="31" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J31" s="2" t="s">
+      <c r="J31" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L31" s="2" t="s">
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" t="s">
         <v>62</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="M31" t="s">
         <v>37</v>
       </c>
-      <c r="O31" s="2">
-        <v>1</v>
-      </c>
-      <c r="P31" s="2" t="s">
+      <c r="O31">
+        <v>1</v>
+      </c>
+      <c r="P31" t="s">
         <v>38</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R31" s="2" t="s">
+      <c r="Q31" t="s">
+        <v>18</v>
+      </c>
+      <c r="R31" t="s">
         <v>47</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31">
         <v>17</v>
       </c>
     </row>
     <row r="32" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J32" s="2" t="s">
+      <c r="J32" t="s">
         <v>65</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L32" s="2" t="s">
+      <c r="K32" t="s">
+        <v>19</v>
+      </c>
+      <c r="L32" t="s">
         <v>62</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" t="s">
         <v>37</v>
       </c>
-      <c r="O32" s="2">
-        <v>1</v>
-      </c>
-      <c r="P32" s="2" t="s">
+      <c r="O32">
+        <v>1</v>
+      </c>
+      <c r="P32" t="s">
         <v>38</v>
       </c>
-      <c r="Q32" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R32" s="2" t="s">
+      <c r="Q32" t="s">
+        <v>18</v>
+      </c>
+      <c r="R32" t="s">
         <v>47</v>
       </c>
-      <c r="T32" s="2">
+      <c r="T32">
         <v>18</v>
       </c>
     </row>
     <row r="33" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J33" s="2" t="s">
+      <c r="J33" t="s">
         <v>66</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="K33" t="s">
+        <v>19</v>
+      </c>
+      <c r="L33" t="s">
         <v>69</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="M33" t="s">
         <v>37</v>
       </c>
-      <c r="O33" s="2">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="s">
+      <c r="O33">
+        <v>1</v>
+      </c>
+      <c r="P33" t="s">
         <v>38</v>
       </c>
-      <c r="Q33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R33" s="2" t="s">
+      <c r="Q33" t="s">
+        <v>18</v>
+      </c>
+      <c r="R33" t="s">
         <v>47</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33">
         <v>19</v>
       </c>
     </row>
     <row r="34" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J34" s="2" t="s">
+      <c r="J34" t="s">
         <v>67</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="K34" t="s">
+        <v>19</v>
+      </c>
+      <c r="L34" t="s">
         <v>68</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" t="s">
         <v>37</v>
       </c>
-      <c r="O34" s="2">
-        <v>1</v>
-      </c>
-      <c r="P34" s="2" t="s">
+      <c r="O34">
+        <v>1</v>
+      </c>
+      <c r="P34" t="s">
         <v>38</v>
       </c>
-      <c r="Q34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R34" s="2" t="s">
+      <c r="Q34" t="s">
+        <v>18</v>
+      </c>
+      <c r="R34" t="s">
         <v>47</v>
       </c>
-      <c r="T34" s="2">
+      <c r="T34">
         <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J35" t="s">
+        <v>74</v>
+      </c>
+      <c r="K35" t="s">
+        <v>18</v>
+      </c>
+      <c r="L35" t="s">
+        <v>76</v>
+      </c>
+      <c r="M35" t="s">
+        <v>37</v>
+      </c>
+      <c r="O35">
+        <v>1</v>
+      </c>
+      <c r="P35" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" t="s">
+        <v>47</v>
+      </c>
+      <c r="T35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J36" t="s">
+        <v>75</v>
+      </c>
+      <c r="K36" t="s">
+        <v>19</v>
+      </c>
+      <c r="L36" t="s">
+        <v>76</v>
+      </c>
+      <c r="M36" t="s">
+        <v>37</v>
+      </c>
+      <c r="O36">
+        <v>1</v>
+      </c>
+      <c r="P36" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>18</v>
+      </c>
+      <c r="R36" t="s">
+        <v>47</v>
+      </c>
+      <c r="T36">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -3660,34 +3714,31 @@
       </c>
     </row>
     <row r="15" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>41</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
         <v>39</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2">
-        <v>1</v>
-      </c>
-      <c r="U15" s="2" t="s">
+      <c r="Q15" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" t="s">
+        <v>22</v>
+      </c>
+      <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3695,7 +3746,7 @@
       <c r="J16" t="s">
         <v>43</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" t="s">
         <v>20</v>
       </c>
       <c r="L16" t="s">
@@ -3704,13 +3755,13 @@
       <c r="O16">
         <v>1</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" t="s">
         <v>39</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="2" t="s">
+      <c r="Q16" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" t="s">
         <v>22</v>
       </c>
       <c r="T16">
@@ -3721,7 +3772,7 @@
       <c r="J17" t="s">
         <v>44</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K17" t="s">
         <v>20</v>
       </c>
       <c r="L17" t="s">
@@ -3730,13 +3781,13 @@
       <c r="O17">
         <v>1</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="P17" t="s">
         <v>39</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R17" s="2" t="s">
+      <c r="Q17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R17" t="s">
         <v>22</v>
       </c>
       <c r="T17">
@@ -3747,7 +3798,7 @@
       <c r="J18" t="s">
         <v>45</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="K18" t="s">
         <v>20</v>
       </c>
       <c r="L18" t="s">
@@ -3756,13 +3807,13 @@
       <c r="O18">
         <v>1</v>
       </c>
-      <c r="P18" s="2" t="s">
+      <c r="P18" t="s">
         <v>39</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R18" s="2" t="s">
+      <c r="Q18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R18" t="s">
         <v>22</v>
       </c>
       <c r="T18">
@@ -3773,7 +3824,7 @@
       <c r="J19" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" t="s">
         <v>20</v>
       </c>
       <c r="L19" t="s">
@@ -3782,13 +3833,13 @@
       <c r="O19">
         <v>1</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="P19" t="s">
         <v>39</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R19" s="2" t="s">
+      <c r="Q19" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" t="s">
         <v>22</v>
       </c>
       <c r="T19">
@@ -3799,7 +3850,7 @@
       <c r="J20" t="s">
         <v>43</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K20" t="s">
         <v>20</v>
       </c>
       <c r="L20" t="s">
@@ -3808,13 +3859,13 @@
       <c r="O20">
         <v>2</v>
       </c>
-      <c r="P20" s="2" t="s">
+      <c r="P20" t="s">
         <v>40</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R20" s="2" t="s">
+      <c r="Q20" t="s">
+        <v>18</v>
+      </c>
+      <c r="R20" t="s">
         <v>22</v>
       </c>
       <c r="T20">
@@ -3825,7 +3876,7 @@
       <c r="J21" t="s">
         <v>44</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" t="s">
         <v>20</v>
       </c>
       <c r="L21" t="s">
@@ -3834,13 +3885,13 @@
       <c r="O21">
         <v>2</v>
       </c>
-      <c r="P21" s="2" t="s">
+      <c r="P21" t="s">
         <v>40</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R21" s="2" t="s">
+      <c r="Q21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R21" t="s">
         <v>22</v>
       </c>
       <c r="T21">
@@ -3851,7 +3902,7 @@
       <c r="J22" t="s">
         <v>45</v>
       </c>
-      <c r="K22" s="2" t="s">
+      <c r="K22" t="s">
         <v>20</v>
       </c>
       <c r="L22" t="s">
@@ -3860,13 +3911,13 @@
       <c r="O22">
         <v>2</v>
       </c>
-      <c r="P22" s="2" t="s">
+      <c r="P22" t="s">
         <v>40</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="Q22" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" t="s">
         <v>22</v>
       </c>
       <c r="T22">
@@ -3877,7 +3928,7 @@
       <c r="J23" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="2" t="s">
+      <c r="K23" t="s">
         <v>20</v>
       </c>
       <c r="L23" t="s">
@@ -3886,13 +3937,13 @@
       <c r="O23">
         <v>2</v>
       </c>
-      <c r="P23" s="2" t="s">
+      <c r="P23" t="s">
         <v>40</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R23" s="2" t="s">
+      <c r="Q23" t="s">
+        <v>18</v>
+      </c>
+      <c r="R23" t="s">
         <v>22</v>
       </c>
       <c r="T23">
@@ -3900,122 +3951,118 @@
       </c>
     </row>
     <row r="24" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>52</v>
       </c>
-      <c r="K24" s="2" t="s">
+      <c r="K24" t="s">
         <v>20</v>
       </c>
-      <c r="L24" s="2" t="s">
+      <c r="L24" t="s">
         <v>56</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" t="s">
         <v>60</v>
       </c>
-      <c r="O24" s="2">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24" t="s">
         <v>38</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R24" s="2" t="s">
+      <c r="Q24" t="s">
+        <v>18</v>
+      </c>
+      <c r="R24" t="s">
         <v>47</v>
       </c>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2">
+      <c r="T24">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>53</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="K25" t="s">
         <v>20</v>
       </c>
-      <c r="L25" s="2" t="s">
+      <c r="L25" t="s">
         <v>57</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" t="s">
         <v>60</v>
       </c>
-      <c r="O25" s="2">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
         <v>38</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R25" s="2" t="s">
+      <c r="Q25" t="s">
+        <v>18</v>
+      </c>
+      <c r="R25" t="s">
         <v>47</v>
       </c>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2">
+      <c r="T25">
         <v>25</v>
       </c>
     </row>
     <row r="26" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>54</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K26" t="s">
         <v>20</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="L26" t="s">
         <v>58</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" t="s">
         <v>60</v>
       </c>
-      <c r="O26" s="2">
-        <v>1</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26">
+        <v>1</v>
+      </c>
+      <c r="P26" t="s">
         <v>38</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R26" s="2" t="s">
+      <c r="Q26" t="s">
+        <v>18</v>
+      </c>
+      <c r="R26" t="s">
         <v>47</v>
       </c>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2">
+      <c r="T26">
         <v>26</v>
       </c>
     </row>
     <row r="27" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>55</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K27" t="s">
         <v>20</v>
       </c>
-      <c r="L27" s="2" t="s">
+      <c r="L27" t="s">
         <v>59</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" t="s">
         <v>60</v>
       </c>
-      <c r="O27" s="2">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
         <v>38</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="Q27" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" t="s">
         <v>47</v>
       </c>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2">
+      <c r="T27">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CASM-5723 - Add support for bare metal fabric manager nodes (#746)
* CASM-5723 - Update CANU to support bare-metal fabric manager

* Update SLS to ensure FMN node addition to service objects ACLs is covered by tests

* Update golden config CCJ file with fmn nodes

* Update SLS file with fmn-vip to ensure NMN isolation ACL generation is correct

* Fix linting error
</commit_message>
<xml_diff>
--- a/tests/data/Full_Architecture_Golden_Config_1.1.5.xlsx
+++ b/tests/data/Full_Architecture_Golden_Config_1.1.5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasbates/canu-container/canu/tests/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cspiller/tickets/CASM-5723/canu_src/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100FBE82-86D9-0640-A3A1-B346532A1D08}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A2A660-5375-DF41-AE22-FD8859523E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="78080" yWindow="2140" windowWidth="28800" windowHeight="17500" xr2:uid="{4E3EDB71-9423-764F-AB16-D8E153A84166}"/>
+    <workbookView xWindow="20" yWindow="620" windowWidth="51200" windowHeight="28180" activeTab="1" xr2:uid="{4E3EDB71-9423-764F-AB16-D8E153A84166}"/>
   </bookViews>
   <sheets>
     <sheet name="SWITCH_TO_SWITCH" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="77">
   <si>
     <t>Source</t>
   </si>
@@ -259,6 +259,15 @@
   </si>
   <si>
     <t>u19</t>
+  </si>
+  <si>
+    <t>fmn01</t>
+  </si>
+  <si>
+    <t>fmn02</t>
+  </si>
+  <si>
+    <t>u20</t>
   </si>
 </sst>
 </file>
@@ -385,10 +394,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -419,9 +427,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -459,7 +467,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -565,7 +573,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -707,7 +715,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -754,24 +762,22 @@
       </c>
     </row>
     <row r="15" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>31</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
         <v>21</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
+      <c r="O15">
         <v>32</v>
       </c>
-      <c r="P15" s="2" t="s">
+      <c r="P15" t="s">
         <v>32</v>
       </c>
-      <c r="Q15" s="2" t="s">
+      <c r="Q15" t="s">
         <v>19</v>
       </c>
       <c r="R15" t="s">
@@ -785,24 +791,22 @@
       </c>
     </row>
     <row r="16" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>31</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" t="s">
         <v>21</v>
       </c>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2">
+      <c r="O16">
         <v>31</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" t="s">
         <v>32</v>
       </c>
-      <c r="Q16" s="2" t="s">
+      <c r="Q16" t="s">
         <v>19</v>
       </c>
       <c r="R16" t="s">
@@ -816,24 +820,22 @@
       </c>
     </row>
     <row r="17" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J17" s="2" t="s">
+      <c r="J17" t="s">
         <v>31</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L17" s="2" t="s">
+      <c r="K17" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2">
+      <c r="O17">
         <v>30</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="P17" t="s">
         <v>32</v>
       </c>
-      <c r="Q17" s="2" t="s">
+      <c r="Q17" t="s">
         <v>19</v>
       </c>
       <c r="R17" t="s">
@@ -847,24 +849,22 @@
       </c>
     </row>
     <row r="18" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J18" s="2" t="s">
+      <c r="J18" t="s">
         <v>31</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="K18" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" t="s">
         <v>21</v>
       </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18" t="s">
         <v>33</v>
       </c>
-      <c r="Q18" s="2" t="s">
+      <c r="Q18" t="s">
         <v>18</v>
       </c>
       <c r="R18" t="s">
@@ -875,24 +875,22 @@
       </c>
     </row>
     <row r="19" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J19" s="2" t="s">
+      <c r="J19" t="s">
         <v>31</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="K19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L19" t="s">
         <v>21</v>
       </c>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2">
-        <v>2</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="O19">
+        <v>2</v>
+      </c>
+      <c r="P19" t="s">
         <v>34</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="Q19" t="s">
         <v>18</v>
       </c>
       <c r="R19" t="s">
@@ -903,24 +901,22 @@
       </c>
     </row>
     <row r="20" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J20" s="2" t="s">
+      <c r="J20" t="s">
         <v>32</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="K20" t="s">
+        <v>19</v>
+      </c>
+      <c r="L20" t="s">
         <v>21</v>
       </c>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2">
-        <v>1</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20" t="s">
         <v>33</v>
       </c>
-      <c r="Q20" s="2" t="s">
+      <c r="Q20" t="s">
         <v>18</v>
       </c>
       <c r="R20" t="s">
@@ -931,24 +927,22 @@
       </c>
     </row>
     <row r="21" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J21" s="2" t="s">
+      <c r="J21" t="s">
         <v>32</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="K21" t="s">
+        <v>19</v>
+      </c>
+      <c r="L21" t="s">
         <v>21</v>
       </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2">
-        <v>2</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="O21">
+        <v>2</v>
+      </c>
+      <c r="P21" t="s">
         <v>34</v>
       </c>
-      <c r="Q21" s="2" t="s">
+      <c r="Q21" t="s">
         <v>18</v>
       </c>
       <c r="R21" t="s">
@@ -959,24 +953,22 @@
       </c>
     </row>
     <row r="22" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J22" s="2" t="s">
+      <c r="J22" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="K22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" t="s">
         <v>21</v>
       </c>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2">
+      <c r="O22">
         <v>3</v>
       </c>
-      <c r="P22" s="2" t="s">
+      <c r="P22" t="s">
         <v>35</v>
       </c>
-      <c r="Q22" s="2" t="s">
+      <c r="Q22" t="s">
         <v>19</v>
       </c>
       <c r="R22" t="s">
@@ -987,24 +979,22 @@
       </c>
     </row>
     <row r="23" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J23" s="2" t="s">
+      <c r="J23" t="s">
         <v>31</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="K23" t="s">
+        <v>18</v>
+      </c>
+      <c r="L23" t="s">
         <v>21</v>
       </c>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2">
+      <c r="O23">
         <v>4</v>
       </c>
-      <c r="P23" s="2" t="s">
+      <c r="P23" t="s">
         <v>36</v>
       </c>
-      <c r="Q23" s="2" t="s">
+      <c r="Q23" t="s">
         <v>19</v>
       </c>
       <c r="R23" t="s">
@@ -1015,24 +1005,22 @@
       </c>
     </row>
     <row r="24" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>32</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="L24" t="s">
         <v>21</v>
       </c>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2">
+      <c r="O24">
         <v>3</v>
       </c>
-      <c r="P24" s="2" t="s">
+      <c r="P24" t="s">
         <v>35</v>
       </c>
-      <c r="Q24" s="2" t="s">
+      <c r="Q24" t="s">
         <v>19</v>
       </c>
       <c r="R24" t="s">
@@ -1043,24 +1031,22 @@
       </c>
     </row>
     <row r="25" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>32</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L25" s="2" t="s">
+      <c r="K25" t="s">
+        <v>19</v>
+      </c>
+      <c r="L25" t="s">
         <v>21</v>
       </c>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2">
+      <c r="O25">
         <v>4</v>
       </c>
-      <c r="P25" s="2" t="s">
+      <c r="P25" t="s">
         <v>36</v>
       </c>
-      <c r="Q25" s="2" t="s">
+      <c r="Q25" t="s">
         <v>19</v>
       </c>
       <c r="R25" t="s">
@@ -1071,24 +1057,22 @@
       </c>
     </row>
     <row r="26" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>33</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2">
+      <c r="K26" t="s">
+        <v>18</v>
+      </c>
+      <c r="L26" t="s">
+        <v>22</v>
+      </c>
+      <c r="O26">
         <v>56</v>
       </c>
-      <c r="P26" s="2" t="s">
+      <c r="P26" t="s">
         <v>34</v>
       </c>
-      <c r="Q26" s="2" t="s">
+      <c r="Q26" t="s">
         <v>18</v>
       </c>
       <c r="R26" t="s">
@@ -1102,24 +1086,22 @@
       </c>
     </row>
     <row r="27" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>33</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2">
+      <c r="K27" t="s">
+        <v>18</v>
+      </c>
+      <c r="L27" t="s">
+        <v>22</v>
+      </c>
+      <c r="O27">
         <v>55</v>
       </c>
-      <c r="P27" s="2" t="s">
+      <c r="P27" t="s">
         <v>34</v>
       </c>
-      <c r="Q27" s="2" t="s">
+      <c r="Q27" t="s">
         <v>18</v>
       </c>
       <c r="R27" t="s">
@@ -1133,24 +1115,22 @@
       </c>
     </row>
     <row r="28" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J28" s="2" t="s">
+      <c r="J28" t="s">
         <v>33</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2">
+      <c r="K28" t="s">
+        <v>18</v>
+      </c>
+      <c r="L28" t="s">
+        <v>22</v>
+      </c>
+      <c r="O28">
         <v>54</v>
       </c>
-      <c r="P28" s="2" t="s">
+      <c r="P28" t="s">
         <v>34</v>
       </c>
-      <c r="Q28" s="2" t="s">
+      <c r="Q28" t="s">
         <v>18</v>
       </c>
       <c r="R28" t="s">
@@ -1164,529 +1144,520 @@
       </c>
     </row>
     <row r="29" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J29" s="2" t="s">
+      <c r="J29" t="s">
         <v>35</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2">
+      <c r="K29" t="s">
+        <v>19</v>
+      </c>
+      <c r="L29" t="s">
+        <v>22</v>
+      </c>
+      <c r="O29">
         <v>56</v>
       </c>
-      <c r="P29" s="2" t="s">
+      <c r="P29" t="s">
         <v>36</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R29" s="2" t="s">
+      <c r="Q29" t="s">
+        <v>19</v>
+      </c>
+      <c r="R29" t="s">
         <v>23</v>
       </c>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2">
+      <c r="T29">
         <v>56</v>
       </c>
-      <c r="U29" s="2" t="s">
+      <c r="U29" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J30" s="2" t="s">
+      <c r="J30" t="s">
         <v>35</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2">
+      <c r="K30" t="s">
+        <v>19</v>
+      </c>
+      <c r="L30" t="s">
+        <v>22</v>
+      </c>
+      <c r="O30">
         <v>55</v>
       </c>
-      <c r="P30" s="2" t="s">
+      <c r="P30" t="s">
         <v>36</v>
       </c>
-      <c r="Q30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R30" s="2" t="s">
+      <c r="Q30" t="s">
+        <v>19</v>
+      </c>
+      <c r="R30" t="s">
         <v>23</v>
       </c>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2">
+      <c r="T30">
         <v>55</v>
       </c>
-      <c r="U30" s="2" t="s">
+      <c r="U30" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J31" s="2" t="s">
+      <c r="J31" t="s">
         <v>35</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2">
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" t="s">
+        <v>22</v>
+      </c>
+      <c r="O31">
         <v>54</v>
       </c>
-      <c r="P31" s="2" t="s">
+      <c r="P31" t="s">
         <v>36</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R31" s="2" t="s">
+      <c r="Q31" t="s">
+        <v>19</v>
+      </c>
+      <c r="R31" t="s">
         <v>23</v>
       </c>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2">
+      <c r="T31">
         <v>54</v>
       </c>
-      <c r="U31" s="2" t="s">
+      <c r="U31" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J32" s="2" t="s">
+      <c r="J32" t="s">
         <v>39</v>
       </c>
-      <c r="K32" s="2" t="s">
+      <c r="K32" t="s">
         <v>20</v>
       </c>
-      <c r="L32" s="2" t="s">
+      <c r="L32" t="s">
         <v>21</v>
       </c>
-      <c r="O32" s="2">
+      <c r="O32">
         <v>52</v>
       </c>
-      <c r="P32" s="2" t="s">
+      <c r="P32" t="s">
         <v>40</v>
       </c>
-      <c r="Q32" s="2" t="s">
+      <c r="Q32" t="s">
         <v>20</v>
       </c>
-      <c r="R32" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T32" s="2">
+      <c r="R32" t="s">
+        <v>22</v>
+      </c>
+      <c r="T32">
         <v>52</v>
       </c>
-      <c r="U32" s="2" t="s">
+      <c r="U32" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J33" s="2" t="s">
+      <c r="J33" t="s">
         <v>39</v>
       </c>
-      <c r="K33" s="2" t="s">
+      <c r="K33" t="s">
         <v>20</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="L33" t="s">
         <v>21</v>
       </c>
-      <c r="O33" s="2">
+      <c r="O33">
         <v>51</v>
       </c>
-      <c r="P33" s="2" t="s">
+      <c r="P33" t="s">
         <v>40</v>
       </c>
-      <c r="Q33" s="2" t="s">
+      <c r="Q33" t="s">
         <v>20</v>
       </c>
-      <c r="R33" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T33" s="2">
+      <c r="R33" t="s">
+        <v>22</v>
+      </c>
+      <c r="T33">
         <v>51</v>
       </c>
-      <c r="U33" s="2" t="s">
+      <c r="U33" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="34" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J34" s="2" t="s">
+      <c r="J34" t="s">
         <v>39</v>
       </c>
-      <c r="K34" s="2" t="s">
+      <c r="K34" t="s">
         <v>20</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L34" t="s">
         <v>21</v>
       </c>
-      <c r="O34" s="2">
+      <c r="O34">
         <v>48</v>
       </c>
-      <c r="P34" s="2" t="s">
+      <c r="P34" t="s">
         <v>40</v>
       </c>
-      <c r="Q34" s="2" t="s">
+      <c r="Q34" t="s">
         <v>20</v>
       </c>
-      <c r="R34" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T34" s="2">
+      <c r="R34" t="s">
+        <v>22</v>
+      </c>
+      <c r="T34">
         <v>48</v>
       </c>
-      <c r="U34" s="2" t="s">
+      <c r="U34" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="35" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J35" s="2" t="s">
+      <c r="J35" t="s">
         <v>39</v>
       </c>
-      <c r="K35" s="2" t="s">
+      <c r="K35" t="s">
         <v>20</v>
       </c>
-      <c r="L35" s="2" t="s">
+      <c r="L35" t="s">
         <v>21</v>
       </c>
-      <c r="O35" s="2">
+      <c r="O35">
         <v>50</v>
       </c>
-      <c r="P35" s="2" t="s">
+      <c r="P35" t="s">
         <v>31</v>
       </c>
-      <c r="Q35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R35" s="2" t="s">
+      <c r="Q35" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" t="s">
         <v>21</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35">
         <v>5</v>
       </c>
     </row>
     <row r="36" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J36" s="2" t="s">
+      <c r="J36" t="s">
         <v>39</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K36" t="s">
         <v>20</v>
       </c>
-      <c r="L36" s="2" t="s">
+      <c r="L36" t="s">
         <v>21</v>
       </c>
-      <c r="O36" s="2">
+      <c r="O36">
         <v>49</v>
       </c>
-      <c r="P36" s="2" t="s">
+      <c r="P36" t="s">
         <v>32</v>
       </c>
-      <c r="Q36" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R36" s="2" t="s">
+      <c r="Q36" t="s">
+        <v>19</v>
+      </c>
+      <c r="R36" t="s">
         <v>21</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36">
         <v>5</v>
       </c>
     </row>
     <row r="37" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J37" s="2" t="s">
+      <c r="J37" t="s">
         <v>40</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="K37" t="s">
         <v>20</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O37" s="2">
+      <c r="L37" t="s">
+        <v>22</v>
+      </c>
+      <c r="O37">
         <v>50</v>
       </c>
-      <c r="P37" s="2" t="s">
+      <c r="P37" t="s">
         <v>31</v>
       </c>
-      <c r="Q37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R37" s="2" t="s">
+      <c r="Q37" t="s">
+        <v>18</v>
+      </c>
+      <c r="R37" t="s">
         <v>21</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37">
         <v>6</v>
       </c>
     </row>
     <row r="38" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J38" s="2" t="s">
+      <c r="J38" t="s">
         <v>40</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="K38" t="s">
         <v>20</v>
       </c>
-      <c r="L38" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O38" s="2">
+      <c r="L38" t="s">
+        <v>22</v>
+      </c>
+      <c r="O38">
         <v>49</v>
       </c>
-      <c r="P38" s="2" t="s">
+      <c r="P38" t="s">
         <v>32</v>
       </c>
-      <c r="Q38" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R38" s="2" t="s">
+      <c r="Q38" t="s">
+        <v>19</v>
+      </c>
+      <c r="R38" t="s">
         <v>21</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38">
         <v>6</v>
       </c>
     </row>
     <row r="39" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J39" s="2" t="s">
+      <c r="J39" t="s">
         <v>49</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="K39" t="s">
         <v>48</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="L39" t="s">
         <v>21</v>
       </c>
-      <c r="O39" s="2">
-        <v>1</v>
-      </c>
-      <c r="P39" s="2" t="s">
+      <c r="O39">
+        <v>1</v>
+      </c>
+      <c r="P39" t="s">
         <v>31</v>
       </c>
-      <c r="Q39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R39" s="2" t="s">
+      <c r="Q39" t="s">
+        <v>18</v>
+      </c>
+      <c r="R39" t="s">
         <v>21</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39">
         <v>7</v>
       </c>
     </row>
     <row r="40" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J40" s="2" t="s">
+      <c r="J40" t="s">
         <v>50</v>
       </c>
-      <c r="K40" s="2" t="s">
+      <c r="K40" t="s">
         <v>48</v>
       </c>
-      <c r="L40" s="2" t="s">
+      <c r="L40" t="s">
         <v>21</v>
       </c>
-      <c r="O40" s="2">
-        <v>1</v>
-      </c>
-      <c r="P40" s="2" t="s">
+      <c r="O40">
+        <v>1</v>
+      </c>
+      <c r="P40" t="s">
         <v>31</v>
       </c>
-      <c r="Q40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R40" s="2" t="s">
+      <c r="Q40" t="s">
+        <v>18</v>
+      </c>
+      <c r="R40" t="s">
         <v>21</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40">
         <v>8</v>
       </c>
     </row>
     <row r="41" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J41" s="2" t="s">
+      <c r="J41" t="s">
         <v>49</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="K41" t="s">
         <v>48</v>
       </c>
-      <c r="L41" s="2" t="s">
+      <c r="L41" t="s">
         <v>21</v>
       </c>
-      <c r="O41" s="2">
-        <v>2</v>
-      </c>
-      <c r="P41" s="2" t="s">
+      <c r="O41">
+        <v>2</v>
+      </c>
+      <c r="P41" t="s">
         <v>32</v>
       </c>
-      <c r="Q41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R41" s="2" t="s">
+      <c r="Q41" t="s">
+        <v>19</v>
+      </c>
+      <c r="R41" t="s">
         <v>21</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41">
         <v>7</v>
       </c>
     </row>
     <row r="42" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J42" s="2" t="s">
+      <c r="J42" t="s">
         <v>50</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="K42" t="s">
         <v>48</v>
       </c>
-      <c r="L42" s="2" t="s">
+      <c r="L42" t="s">
         <v>21</v>
       </c>
-      <c r="O42" s="2">
-        <v>2</v>
-      </c>
-      <c r="P42" s="2" t="s">
+      <c r="O42">
+        <v>2</v>
+      </c>
+      <c r="P42" t="s">
         <v>32</v>
       </c>
-      <c r="Q42" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R42" s="2" t="s">
+      <c r="Q42" t="s">
+        <v>19</v>
+      </c>
+      <c r="R42" t="s">
         <v>21</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42">
         <v>8</v>
       </c>
     </row>
     <row r="43" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J43" s="2" t="s">
+      <c r="J43" t="s">
         <v>38</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L43" s="2" t="s">
+      <c r="K43" t="s">
+        <v>18</v>
+      </c>
+      <c r="L43" t="s">
         <v>47</v>
       </c>
-      <c r="O43" s="2">
+      <c r="O43">
         <v>48</v>
       </c>
-      <c r="P43" s="2" t="s">
+      <c r="P43" t="s">
         <v>33</v>
       </c>
-      <c r="Q43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R43" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T43" s="2">
+      <c r="Q43" t="s">
+        <v>18</v>
+      </c>
+      <c r="R43" t="s">
+        <v>22</v>
+      </c>
+      <c r="T43">
         <v>51</v>
       </c>
     </row>
     <row r="44" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J44" s="2" t="s">
+      <c r="J44" t="s">
         <v>38</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L44" s="2" t="s">
+      <c r="K44" t="s">
+        <v>18</v>
+      </c>
+      <c r="L44" t="s">
         <v>47</v>
       </c>
-      <c r="O44" s="2">
+      <c r="O44">
         <v>47</v>
       </c>
-      <c r="P44" s="2" t="s">
+      <c r="P44" t="s">
         <v>34</v>
       </c>
-      <c r="Q44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R44" s="2" t="s">
+      <c r="Q44" t="s">
+        <v>18</v>
+      </c>
+      <c r="R44" t="s">
         <v>23</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44">
         <v>51</v>
       </c>
     </row>
     <row r="45" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J45" s="3" t="s">
+      <c r="J45" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K45" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L45" s="5" t="s">
+      <c r="K45" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="L45" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="N45" s="6" t="s">
+      <c r="N45" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O45" s="7">
-        <v>1</v>
-      </c>
-      <c r="P45" s="3" t="s">
+      <c r="O45" s="6">
+        <v>1</v>
+      </c>
+      <c r="P45" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Q45" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R45" s="5" t="s">
+      <c r="Q45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R45" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="T45" s="7">
+      <c r="T45" s="6">
         <v>29</v>
       </c>
     </row>
     <row r="46" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J46" s="3" t="s">
+      <c r="J46" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K46" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L46" s="5" t="s">
+      <c r="K46" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="L46" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="N46" s="6" t="s">
+      <c r="N46" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O46" s="7">
-        <v>2</v>
-      </c>
-      <c r="P46" s="3" t="s">
+      <c r="O46" s="6">
+        <v>2</v>
+      </c>
+      <c r="P46" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q46" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R46" s="5" t="s">
+      <c r="Q46" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R46" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T46" s="7">
+      <c r="T46" s="6">
         <v>29</v>
       </c>
     </row>
     <row r="47" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J47" s="3" t="s">
+      <c r="J47" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K47" s="4" t="s">
+      <c r="K47" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L47" t="s">
         <v>73</v>
       </c>
-      <c r="N47" s="6" t="s">
+      <c r="N47" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O47">
         <v>1</v>
       </c>
-      <c r="P47" s="3" t="s">
+      <c r="P47" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Q47" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R47" s="5" t="s">
+      <c r="Q47" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R47" s="4" t="s">
         <v>47</v>
       </c>
       <c r="T47">
@@ -1694,28 +1665,28 @@
       </c>
     </row>
     <row r="48" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J48" s="3" t="s">
+      <c r="J48" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K48" s="4" t="s">
+      <c r="K48" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L48" t="s">
         <v>73</v>
       </c>
-      <c r="N48" s="6" t="s">
+      <c r="N48" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O48">
         <v>2</v>
       </c>
-      <c r="P48" s="3" t="s">
+      <c r="P48" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="Q48" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="R48" s="5" t="s">
+      <c r="Q48" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="R48" s="4" t="s">
         <v>23</v>
       </c>
       <c r="T48">
@@ -1729,7 +1700,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6C3018C-CE0C-E04E-8947-8C874399EC7B}">
-  <dimension ref="J14:T53"/>
+  <dimension ref="J14:T57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -1770,1202 +1741,1250 @@
       </c>
     </row>
     <row r="15" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="M15" t="s">
         <v>16</v>
       </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
         <v>33</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2">
+      <c r="Q15" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" t="s">
+        <v>22</v>
+      </c>
+      <c r="T15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>6</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" t="s">
         <v>24</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M16" t="s">
         <v>16</v>
       </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2">
-        <v>2</v>
-      </c>
-      <c r="P16" s="2" t="s">
+      <c r="O16">
+        <v>2</v>
+      </c>
+      <c r="P16" t="s">
         <v>51</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2">
+      <c r="Q16" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" t="s">
+        <v>22</v>
+      </c>
+      <c r="T16">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J17" s="2" t="s">
+      <c r="J17" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L17" s="2" t="s">
+      <c r="K17" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" t="s">
         <v>24</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M17" t="s">
         <v>17</v>
       </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="s">
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17" t="s">
         <v>34</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R17" s="2" t="s">
+      <c r="Q17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R17" t="s">
         <v>23</v>
       </c>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2">
+      <c r="T17">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J18" s="2" t="s">
+      <c r="J18" t="s">
         <v>6</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="K18" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" t="s">
         <v>24</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M18" t="s">
         <v>17</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2">
-        <v>2</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="O18">
+        <v>2</v>
+      </c>
+      <c r="P18" t="s">
         <v>51</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R18" s="2" t="s">
+      <c r="Q18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R18" t="s">
         <v>23</v>
       </c>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2">
+      <c r="T18">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J19" s="2" t="s">
+      <c r="J19" t="s">
         <v>7</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="K19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L19" t="s">
         <v>25</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" t="s">
         <v>16</v>
       </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2">
-        <v>1</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19" t="s">
         <v>33</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R19" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2">
+      <c r="Q19" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" t="s">
+        <v>22</v>
+      </c>
+      <c r="T19">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J20" s="2" t="s">
+      <c r="J20" t="s">
         <v>7</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="K20" t="s">
+        <v>18</v>
+      </c>
+      <c r="L20" t="s">
         <v>25</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="M20" t="s">
         <v>16</v>
       </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2">
-        <v>2</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20">
+        <v>2</v>
+      </c>
+      <c r="P20" t="s">
         <v>51</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2">
+      <c r="Q20" t="s">
+        <v>18</v>
+      </c>
+      <c r="R20" t="s">
+        <v>22</v>
+      </c>
+      <c r="T20">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J21" s="2" t="s">
+      <c r="J21" t="s">
         <v>7</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="K21" t="s">
+        <v>18</v>
+      </c>
+      <c r="L21" t="s">
         <v>25</v>
       </c>
-      <c r="M21" s="2" t="s">
+      <c r="M21" t="s">
         <v>17</v>
       </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21" t="s">
         <v>34</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R21" s="2" t="s">
+      <c r="Q21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R21" t="s">
         <v>23</v>
       </c>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2">
+      <c r="T21">
         <v>3</v>
       </c>
     </row>
     <row r="22" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J22" s="2" t="s">
+      <c r="J22" t="s">
         <v>7</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="K22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" t="s">
         <v>25</v>
       </c>
-      <c r="M22" s="2" t="s">
+      <c r="M22" t="s">
         <v>17</v>
       </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2">
-        <v>2</v>
-      </c>
-      <c r="P22" s="2" t="s">
+      <c r="O22">
+        <v>2</v>
+      </c>
+      <c r="P22" t="s">
         <v>51</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="Q22" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" t="s">
         <v>23</v>
       </c>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2">
+      <c r="T22">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J23" s="2" t="s">
+      <c r="J23" t="s">
         <v>8</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="K23" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" t="s">
         <v>24</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="M23" t="s">
         <v>16</v>
       </c>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2">
-        <v>1</v>
-      </c>
-      <c r="P23" s="2" t="s">
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23" t="s">
         <v>35</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2">
+      <c r="Q23" t="s">
+        <v>19</v>
+      </c>
+      <c r="R23" t="s">
+        <v>22</v>
+      </c>
+      <c r="T23">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>8</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="L24" t="s">
         <v>24</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" t="s">
         <v>16</v>
       </c>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2">
-        <v>2</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="O24">
+        <v>2</v>
+      </c>
+      <c r="P24" t="s">
         <v>51</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2">
+      <c r="Q24" t="s">
+        <v>19</v>
+      </c>
+      <c r="R24" t="s">
+        <v>22</v>
+      </c>
+      <c r="T24">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>8</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L25" s="2" t="s">
+      <c r="K25" t="s">
+        <v>19</v>
+      </c>
+      <c r="L25" t="s">
         <v>24</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" t="s">
         <v>17</v>
       </c>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
         <v>36</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R25" s="2" t="s">
+      <c r="Q25" t="s">
+        <v>19</v>
+      </c>
+      <c r="R25" t="s">
         <v>23</v>
       </c>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2">
+      <c r="T25">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>8</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L26" s="2" t="s">
+      <c r="K26" t="s">
+        <v>19</v>
+      </c>
+      <c r="L26" t="s">
         <v>24</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" t="s">
         <v>17</v>
       </c>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2">
-        <v>2</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26">
+        <v>2</v>
+      </c>
+      <c r="P26" t="s">
         <v>51</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R26" s="2" t="s">
+      <c r="Q26" t="s">
+        <v>19</v>
+      </c>
+      <c r="R26" t="s">
         <v>23</v>
       </c>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2">
+      <c r="T26">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>9</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L27" s="2" t="s">
+      <c r="K27" t="s">
+        <v>18</v>
+      </c>
+      <c r="L27" t="s">
         <v>26</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" t="s">
         <v>16</v>
       </c>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
         <v>33</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R27" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2">
+      <c r="Q27" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" t="s">
+        <v>22</v>
+      </c>
+      <c r="T27">
         <v>5</v>
       </c>
     </row>
     <row r="28" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J28" s="2" t="s">
+      <c r="J28" t="s">
         <v>9</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L28" s="2" t="s">
+      <c r="K28" t="s">
+        <v>18</v>
+      </c>
+      <c r="L28" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" t="s">
         <v>16</v>
       </c>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2">
-        <v>2</v>
-      </c>
-      <c r="P28" s="2" t="s">
+      <c r="O28">
+        <v>2</v>
+      </c>
+      <c r="P28" t="s">
         <v>34</v>
       </c>
-      <c r="Q28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R28" s="2" t="s">
+      <c r="Q28" t="s">
+        <v>18</v>
+      </c>
+      <c r="R28" t="s">
         <v>23</v>
       </c>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2">
+      <c r="T28">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J29" s="2" t="s">
+      <c r="J29" t="s">
         <v>10</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L29" s="2" t="s">
+      <c r="K29" t="s">
+        <v>19</v>
+      </c>
+      <c r="L29" t="s">
         <v>25</v>
       </c>
-      <c r="M29" s="2" t="s">
+      <c r="M29" t="s">
         <v>16</v>
       </c>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2">
-        <v>1</v>
-      </c>
-      <c r="P29" s="2" t="s">
+      <c r="O29">
+        <v>1</v>
+      </c>
+      <c r="P29" t="s">
         <v>35</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S29" s="2"/>
-      <c r="T29" s="2">
+      <c r="Q29" t="s">
+        <v>19</v>
+      </c>
+      <c r="R29" t="s">
+        <v>22</v>
+      </c>
+      <c r="T29">
         <v>3</v>
       </c>
     </row>
     <row r="30" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J30" s="2" t="s">
+      <c r="J30" t="s">
         <v>10</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L30" s="2" t="s">
+      <c r="K30" t="s">
+        <v>19</v>
+      </c>
+      <c r="L30" t="s">
         <v>25</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="M30" t="s">
         <v>16</v>
       </c>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2">
-        <v>2</v>
-      </c>
-      <c r="P30" s="2" t="s">
+      <c r="O30">
+        <v>2</v>
+      </c>
+      <c r="P30" t="s">
         <v>36</v>
       </c>
-      <c r="Q30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R30" s="2" t="s">
+      <c r="Q30" t="s">
+        <v>19</v>
+      </c>
+      <c r="R30" t="s">
         <v>23</v>
       </c>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2">
+      <c r="T30">
         <v>3</v>
       </c>
     </row>
     <row r="31" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J31" s="2" t="s">
+      <c r="J31" t="s">
         <v>11</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L31" s="2" t="s">
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" t="s">
         <v>26</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="M31" t="s">
         <v>16</v>
       </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2">
-        <v>1</v>
-      </c>
-      <c r="P31" s="2" t="s">
+      <c r="O31">
+        <v>1</v>
+      </c>
+      <c r="P31" t="s">
         <v>35</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R31" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2">
+      <c r="Q31" t="s">
+        <v>19</v>
+      </c>
+      <c r="R31" t="s">
+        <v>22</v>
+      </c>
+      <c r="T31">
         <v>4</v>
       </c>
     </row>
     <row r="32" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J32" s="2" t="s">
+      <c r="J32" t="s">
         <v>11</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L32" s="2" t="s">
+      <c r="K32" t="s">
+        <v>19</v>
+      </c>
+      <c r="L32" t="s">
         <v>26</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" t="s">
         <v>16</v>
       </c>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2">
-        <v>2</v>
-      </c>
-      <c r="P32" s="2" t="s">
+      <c r="O32">
+        <v>2</v>
+      </c>
+      <c r="P32" t="s">
         <v>36</v>
       </c>
-      <c r="Q32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R32" s="2" t="s">
+      <c r="Q32" t="s">
+        <v>19</v>
+      </c>
+      <c r="R32" t="s">
         <v>23</v>
       </c>
-      <c r="S32" s="2"/>
-      <c r="T32" s="2">
+      <c r="T32">
         <v>4</v>
       </c>
     </row>
     <row r="33" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J33" s="2" t="s">
+      <c r="J33" t="s">
         <v>12</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="K33" t="s">
+        <v>18</v>
+      </c>
+      <c r="L33" t="s">
         <v>27</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="M33" t="s">
         <v>16</v>
       </c>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="s">
+      <c r="O33">
+        <v>1</v>
+      </c>
+      <c r="P33" t="s">
         <v>33</v>
       </c>
-      <c r="Q33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S33" s="2"/>
-      <c r="T33" s="2">
+      <c r="Q33" t="s">
+        <v>18</v>
+      </c>
+      <c r="R33" t="s">
+        <v>22</v>
+      </c>
+      <c r="T33">
         <v>7</v>
       </c>
     </row>
     <row r="34" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J34" s="2" t="s">
+      <c r="J34" t="s">
         <v>12</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="K34" t="s">
+        <v>18</v>
+      </c>
+      <c r="L34" t="s">
         <v>27</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" t="s">
         <v>16</v>
       </c>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2">
-        <v>2</v>
-      </c>
-      <c r="P34" s="2" t="s">
+      <c r="O34">
+        <v>2</v>
+      </c>
+      <c r="P34" t="s">
         <v>33</v>
       </c>
-      <c r="Q34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R34" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S34" s="2"/>
-      <c r="T34" s="2">
+      <c r="Q34" t="s">
+        <v>18</v>
+      </c>
+      <c r="R34" t="s">
+        <v>22</v>
+      </c>
+      <c r="T34">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J35" s="2" t="s">
+      <c r="J35" t="s">
         <v>12</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L35" s="2" t="s">
+      <c r="K35" t="s">
+        <v>18</v>
+      </c>
+      <c r="L35" t="s">
         <v>27</v>
       </c>
-      <c r="M35" s="2" t="s">
+      <c r="M35" t="s">
         <v>17</v>
       </c>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2">
-        <v>1</v>
-      </c>
-      <c r="P35" s="2" t="s">
+      <c r="O35">
+        <v>1</v>
+      </c>
+      <c r="P35" t="s">
         <v>34</v>
       </c>
-      <c r="Q35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R35" s="2" t="s">
+      <c r="Q35" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" t="s">
         <v>23</v>
       </c>
-      <c r="S35" s="2"/>
-      <c r="T35" s="2">
+      <c r="T35">
         <v>7</v>
       </c>
     </row>
     <row r="36" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J36" s="2" t="s">
+      <c r="J36" t="s">
         <v>12</v>
       </c>
-      <c r="K36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L36" s="2" t="s">
+      <c r="K36" t="s">
+        <v>18</v>
+      </c>
+      <c r="L36" t="s">
         <v>27</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="M36" t="s">
         <v>17</v>
       </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2">
-        <v>2</v>
-      </c>
-      <c r="P36" s="2" t="s">
+      <c r="O36">
+        <v>2</v>
+      </c>
+      <c r="P36" t="s">
         <v>34</v>
       </c>
-      <c r="Q36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R36" s="2" t="s">
+      <c r="Q36" t="s">
+        <v>18</v>
+      </c>
+      <c r="R36" t="s">
         <v>23</v>
       </c>
-      <c r="S36" s="2"/>
-      <c r="T36" s="2">
+      <c r="T36">
         <v>8</v>
       </c>
     </row>
     <row r="37" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J37" s="2" t="s">
+      <c r="J37" t="s">
         <v>13</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L37" s="2" t="s">
+      <c r="K37" t="s">
+        <v>18</v>
+      </c>
+      <c r="L37" t="s">
         <v>28</v>
       </c>
-      <c r="M37" s="2" t="s">
+      <c r="M37" t="s">
         <v>16</v>
       </c>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2">
-        <v>1</v>
-      </c>
-      <c r="P37" s="2" t="s">
+      <c r="O37">
+        <v>1</v>
+      </c>
+      <c r="P37" t="s">
         <v>33</v>
       </c>
-      <c r="Q37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R37" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S37" s="2"/>
-      <c r="T37" s="2">
+      <c r="Q37" t="s">
+        <v>18</v>
+      </c>
+      <c r="R37" t="s">
+        <v>22</v>
+      </c>
+      <c r="T37">
         <v>9</v>
       </c>
     </row>
     <row r="38" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J38" s="2" t="s">
+      <c r="J38" t="s">
         <v>13</v>
       </c>
-      <c r="K38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L38" s="2" t="s">
+      <c r="K38" t="s">
+        <v>18</v>
+      </c>
+      <c r="L38" t="s">
         <v>28</v>
       </c>
-      <c r="M38" s="2" t="s">
+      <c r="M38" t="s">
         <v>16</v>
       </c>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2">
-        <v>2</v>
-      </c>
-      <c r="P38" s="2" t="s">
+      <c r="O38">
+        <v>2</v>
+      </c>
+      <c r="P38" t="s">
         <v>33</v>
       </c>
-      <c r="Q38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R38" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S38" s="2"/>
-      <c r="T38" s="2">
+      <c r="Q38" t="s">
+        <v>18</v>
+      </c>
+      <c r="R38" t="s">
+        <v>22</v>
+      </c>
+      <c r="T38">
         <v>10</v>
       </c>
     </row>
     <row r="39" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J39" s="2" t="s">
+      <c r="J39" t="s">
         <v>13</v>
       </c>
-      <c r="K39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L39" s="2" t="s">
+      <c r="K39" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" t="s">
         <v>28</v>
       </c>
-      <c r="M39" s="2" t="s">
+      <c r="M39" t="s">
         <v>17</v>
       </c>
-      <c r="N39" s="2"/>
-      <c r="O39" s="2">
-        <v>1</v>
-      </c>
-      <c r="P39" s="2" t="s">
+      <c r="O39">
+        <v>1</v>
+      </c>
+      <c r="P39" t="s">
         <v>34</v>
       </c>
-      <c r="Q39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R39" s="2" t="s">
+      <c r="Q39" t="s">
+        <v>18</v>
+      </c>
+      <c r="R39" t="s">
         <v>23</v>
       </c>
-      <c r="S39" s="2"/>
-      <c r="T39" s="2">
+      <c r="T39">
         <v>9</v>
       </c>
     </row>
     <row r="40" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J40" s="2" t="s">
+      <c r="J40" t="s">
         <v>13</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L40" s="2" t="s">
+      <c r="K40" t="s">
+        <v>18</v>
+      </c>
+      <c r="L40" t="s">
         <v>28</v>
       </c>
-      <c r="M40" s="2" t="s">
+      <c r="M40" t="s">
         <v>17</v>
       </c>
-      <c r="N40" s="2"/>
-      <c r="O40" s="2">
-        <v>2</v>
-      </c>
-      <c r="P40" s="2" t="s">
+      <c r="O40">
+        <v>2</v>
+      </c>
+      <c r="P40" t="s">
         <v>34</v>
       </c>
-      <c r="Q40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R40" s="2" t="s">
+      <c r="Q40" t="s">
+        <v>18</v>
+      </c>
+      <c r="R40" t="s">
         <v>23</v>
       </c>
-      <c r="S40" s="2"/>
-      <c r="T40" s="2">
+      <c r="T40">
         <v>10</v>
       </c>
     </row>
     <row r="41" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J41" s="2" t="s">
+      <c r="J41" t="s">
         <v>14</v>
       </c>
-      <c r="K41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L41" s="2" t="s">
+      <c r="K41" t="s">
+        <v>19</v>
+      </c>
+      <c r="L41" t="s">
         <v>27</v>
       </c>
-      <c r="M41" s="2" t="s">
+      <c r="M41" t="s">
         <v>16</v>
       </c>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2">
-        <v>1</v>
-      </c>
-      <c r="P41" s="2" t="s">
+      <c r="O41">
+        <v>1</v>
+      </c>
+      <c r="P41" t="s">
         <v>35</v>
       </c>
-      <c r="Q41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R41" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S41" s="2"/>
-      <c r="T41" s="2">
+      <c r="Q41" t="s">
+        <v>19</v>
+      </c>
+      <c r="R41" t="s">
+        <v>22</v>
+      </c>
+      <c r="T41">
         <v>5</v>
       </c>
     </row>
     <row r="42" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J42" s="2" t="s">
+      <c r="J42" t="s">
         <v>14</v>
       </c>
-      <c r="K42" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L42" s="2" t="s">
+      <c r="K42" t="s">
+        <v>19</v>
+      </c>
+      <c r="L42" t="s">
         <v>27</v>
       </c>
-      <c r="M42" s="2" t="s">
+      <c r="M42" t="s">
         <v>16</v>
       </c>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2">
-        <v>2</v>
-      </c>
-      <c r="P42" s="2" t="s">
+      <c r="O42">
+        <v>2</v>
+      </c>
+      <c r="P42" t="s">
         <v>35</v>
       </c>
-      <c r="Q42" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R42" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S42" s="2"/>
-      <c r="T42" s="2">
+      <c r="Q42" t="s">
+        <v>19</v>
+      </c>
+      <c r="R42" t="s">
+        <v>22</v>
+      </c>
+      <c r="T42">
         <v>6</v>
       </c>
     </row>
     <row r="43" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J43" s="2" t="s">
+      <c r="J43" t="s">
         <v>14</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L43" s="2" t="s">
+      <c r="K43" t="s">
+        <v>19</v>
+      </c>
+      <c r="L43" t="s">
         <v>27</v>
       </c>
-      <c r="M43" s="2" t="s">
+      <c r="M43" t="s">
         <v>17</v>
       </c>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2">
-        <v>1</v>
-      </c>
-      <c r="P43" s="2" t="s">
+      <c r="O43">
+        <v>1</v>
+      </c>
+      <c r="P43" t="s">
         <v>36</v>
       </c>
-      <c r="Q43" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R43" s="2" t="s">
+      <c r="Q43" t="s">
+        <v>19</v>
+      </c>
+      <c r="R43" t="s">
         <v>23</v>
       </c>
-      <c r="S43" s="2"/>
-      <c r="T43" s="2">
+      <c r="T43">
         <v>5</v>
       </c>
     </row>
     <row r="44" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J44" s="2" t="s">
+      <c r="J44" t="s">
         <v>14</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L44" s="2" t="s">
+      <c r="K44" t="s">
+        <v>19</v>
+      </c>
+      <c r="L44" t="s">
         <v>27</v>
       </c>
-      <c r="M44" s="2" t="s">
+      <c r="M44" t="s">
         <v>17</v>
       </c>
-      <c r="N44" s="2"/>
-      <c r="O44" s="2">
-        <v>2</v>
-      </c>
-      <c r="P44" s="2" t="s">
+      <c r="O44">
+        <v>2</v>
+      </c>
+      <c r="P44" t="s">
         <v>36</v>
       </c>
-      <c r="Q44" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R44" s="2" t="s">
+      <c r="Q44" t="s">
+        <v>19</v>
+      </c>
+      <c r="R44" t="s">
         <v>23</v>
       </c>
-      <c r="S44" s="2"/>
-      <c r="T44" s="2">
+      <c r="T44">
         <v>6</v>
       </c>
     </row>
     <row r="45" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J45" s="2" t="s">
+      <c r="J45" t="s">
         <v>15</v>
       </c>
-      <c r="K45" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L45" s="2" t="s">
+      <c r="K45" t="s">
+        <v>19</v>
+      </c>
+      <c r="L45" t="s">
         <v>28</v>
       </c>
-      <c r="M45" s="2" t="s">
+      <c r="M45" t="s">
         <v>16</v>
       </c>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2">
-        <v>1</v>
-      </c>
-      <c r="P45" s="2" t="s">
+      <c r="O45">
+        <v>1</v>
+      </c>
+      <c r="P45" t="s">
         <v>35</v>
       </c>
-      <c r="Q45" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R45" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2">
+      <c r="Q45" t="s">
+        <v>19</v>
+      </c>
+      <c r="R45" t="s">
+        <v>22</v>
+      </c>
+      <c r="T45">
         <v>7</v>
       </c>
     </row>
     <row r="46" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J46" s="2" t="s">
+      <c r="J46" t="s">
         <v>15</v>
       </c>
-      <c r="K46" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L46" s="2" t="s">
+      <c r="K46" t="s">
+        <v>19</v>
+      </c>
+      <c r="L46" t="s">
         <v>28</v>
       </c>
-      <c r="M46" s="2" t="s">
+      <c r="M46" t="s">
         <v>16</v>
       </c>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2">
-        <v>2</v>
-      </c>
-      <c r="P46" s="2" t="s">
+      <c r="O46">
+        <v>2</v>
+      </c>
+      <c r="P46" t="s">
         <v>35</v>
       </c>
-      <c r="Q46" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R46" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S46" s="2"/>
-      <c r="T46" s="2">
+      <c r="Q46" t="s">
+        <v>19</v>
+      </c>
+      <c r="R46" t="s">
+        <v>22</v>
+      </c>
+      <c r="T46">
         <v>8</v>
       </c>
     </row>
     <row r="47" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J47" s="2" t="s">
+      <c r="J47" t="s">
         <v>15</v>
       </c>
-      <c r="K47" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L47" s="2" t="s">
+      <c r="K47" t="s">
+        <v>19</v>
+      </c>
+      <c r="L47" t="s">
         <v>28</v>
       </c>
-      <c r="M47" s="2" t="s">
+      <c r="M47" t="s">
         <v>17</v>
       </c>
-      <c r="N47" s="2"/>
-      <c r="O47" s="2">
-        <v>1</v>
-      </c>
-      <c r="P47" s="2" t="s">
+      <c r="O47">
+        <v>1</v>
+      </c>
+      <c r="P47" t="s">
         <v>36</v>
       </c>
-      <c r="Q47" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R47" s="2" t="s">
+      <c r="Q47" t="s">
+        <v>19</v>
+      </c>
+      <c r="R47" t="s">
         <v>23</v>
       </c>
-      <c r="S47" s="2"/>
-      <c r="T47" s="2">
+      <c r="T47">
         <v>7</v>
       </c>
     </row>
     <row r="48" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J48" s="2" t="s">
+      <c r="J48" t="s">
         <v>15</v>
       </c>
-      <c r="K48" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L48" s="2" t="s">
+      <c r="K48" t="s">
+        <v>19</v>
+      </c>
+      <c r="L48" t="s">
         <v>28</v>
       </c>
-      <c r="M48" s="2" t="s">
+      <c r="M48" t="s">
         <v>17</v>
       </c>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2">
-        <v>2</v>
-      </c>
-      <c r="P48" s="2" t="s">
+      <c r="O48">
+        <v>2</v>
+      </c>
+      <c r="P48" t="s">
         <v>36</v>
       </c>
-      <c r="Q48" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R48" s="2" t="s">
+      <c r="Q48" t="s">
+        <v>19</v>
+      </c>
+      <c r="R48" t="s">
         <v>23</v>
       </c>
-      <c r="S48" s="2"/>
-      <c r="T48" s="2">
+      <c r="T48">
         <v>8</v>
       </c>
     </row>
     <row r="49" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J49" s="2" t="s">
+      <c r="J49" t="s">
         <v>67</v>
       </c>
-      <c r="K49" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L49" s="2" t="s">
+      <c r="K49" t="s">
+        <v>19</v>
+      </c>
+      <c r="L49" t="s">
         <v>68</v>
       </c>
-      <c r="M49" s="2" t="s">
+      <c r="M49" t="s">
         <v>16</v>
       </c>
-      <c r="O49" s="2">
-        <v>1</v>
-      </c>
-      <c r="P49" s="2" t="s">
+      <c r="O49">
+        <v>1</v>
+      </c>
+      <c r="P49" t="s">
         <v>35</v>
       </c>
-      <c r="Q49" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R49" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T49" s="2">
+      <c r="Q49" t="s">
+        <v>19</v>
+      </c>
+      <c r="R49" t="s">
+        <v>22</v>
+      </c>
+      <c r="T49">
         <v>9</v>
       </c>
     </row>
     <row r="50" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J50" s="2" t="s">
+      <c r="J50" t="s">
         <v>67</v>
       </c>
-      <c r="K50" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L50" s="2" t="s">
+      <c r="K50" t="s">
+        <v>19</v>
+      </c>
+      <c r="L50" t="s">
         <v>68</v>
       </c>
-      <c r="M50" s="2" t="s">
+      <c r="M50" t="s">
         <v>16</v>
       </c>
-      <c r="O50" s="2">
-        <v>2</v>
-      </c>
-      <c r="P50" s="2" t="s">
+      <c r="O50">
+        <v>2</v>
+      </c>
+      <c r="P50" t="s">
         <v>35</v>
       </c>
-      <c r="Q50" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R50" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T50" s="2">
+      <c r="Q50" t="s">
+        <v>19</v>
+      </c>
+      <c r="R50" t="s">
+        <v>22</v>
+      </c>
+      <c r="T50">
         <v>10</v>
       </c>
     </row>
     <row r="51" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J51" s="2" t="s">
+      <c r="J51" t="s">
         <v>67</v>
       </c>
-      <c r="K51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L51" s="2" t="s">
+      <c r="K51" t="s">
+        <v>19</v>
+      </c>
+      <c r="L51" t="s">
         <v>68</v>
       </c>
-      <c r="M51" s="2" t="s">
+      <c r="M51" t="s">
         <v>17</v>
       </c>
-      <c r="O51" s="2">
-        <v>1</v>
-      </c>
-      <c r="P51" s="2" t="s">
+      <c r="O51">
+        <v>1</v>
+      </c>
+      <c r="P51" t="s">
         <v>36</v>
       </c>
-      <c r="Q51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R51" s="2" t="s">
+      <c r="Q51" t="s">
+        <v>19</v>
+      </c>
+      <c r="R51" t="s">
         <v>23</v>
       </c>
-      <c r="T51" s="2">
+      <c r="T51">
         <v>9</v>
       </c>
     </row>
     <row r="52" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J52" s="2" t="s">
+      <c r="J52" t="s">
         <v>67</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L52" s="2" t="s">
+      <c r="K52" t="s">
+        <v>19</v>
+      </c>
+      <c r="L52" t="s">
         <v>68</v>
       </c>
-      <c r="M52" s="2" t="s">
+      <c r="M52" t="s">
         <v>17</v>
       </c>
-      <c r="O52" s="2">
-        <v>2</v>
-      </c>
-      <c r="P52" s="2" t="s">
+      <c r="O52">
+        <v>2</v>
+      </c>
+      <c r="P52" t="s">
         <v>36</v>
       </c>
-      <c r="Q52" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="R52" s="2" t="s">
+      <c r="Q52" t="s">
+        <v>19</v>
+      </c>
+      <c r="R52" t="s">
         <v>23</v>
       </c>
-      <c r="T52" s="2">
+      <c r="T52">
         <v>10</v>
       </c>
     </row>
     <row r="53" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J53" s="2" t="s">
+      <c r="J53" t="s">
         <v>66</v>
       </c>
-      <c r="K53" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L53" s="2" t="s">
+      <c r="K53" t="s">
+        <v>19</v>
+      </c>
+      <c r="L53" t="s">
         <v>68</v>
       </c>
-      <c r="M53" s="2" t="s">
+      <c r="M53" t="s">
         <v>16</v>
       </c>
-      <c r="O53" s="2">
-        <v>1</v>
-      </c>
-      <c r="P53" s="2" t="s">
+      <c r="O53">
+        <v>1</v>
+      </c>
+      <c r="P53" t="s">
         <v>38</v>
       </c>
-      <c r="Q53" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R53" s="2" t="s">
+      <c r="Q53" t="s">
+        <v>18</v>
+      </c>
+      <c r="R53" t="s">
         <v>47</v>
       </c>
-      <c r="T53" s="2">
+      <c r="T53">
         <v>28</v>
+      </c>
+    </row>
+    <row r="54" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J54" t="s">
+        <v>74</v>
+      </c>
+      <c r="K54" t="s">
+        <v>18</v>
+      </c>
+      <c r="L54" t="s">
+        <v>76</v>
+      </c>
+      <c r="M54" t="s">
+        <v>16</v>
+      </c>
+      <c r="O54">
+        <v>1</v>
+      </c>
+      <c r="P54" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>18</v>
+      </c>
+      <c r="R54" t="s">
+        <v>22</v>
+      </c>
+      <c r="T54">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J55" t="s">
+        <v>74</v>
+      </c>
+      <c r="K55" t="s">
+        <v>18</v>
+      </c>
+      <c r="L55" t="s">
+        <v>76</v>
+      </c>
+      <c r="M55" t="s">
+        <v>16</v>
+      </c>
+      <c r="O55">
+        <v>2</v>
+      </c>
+      <c r="P55" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>18</v>
+      </c>
+      <c r="R55" t="s">
+        <v>23</v>
+      </c>
+      <c r="T55">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J56" t="s">
+        <v>75</v>
+      </c>
+      <c r="K56" t="s">
+        <v>19</v>
+      </c>
+      <c r="L56" t="s">
+        <v>76</v>
+      </c>
+      <c r="M56" t="s">
+        <v>16</v>
+      </c>
+      <c r="O56">
+        <v>1</v>
+      </c>
+      <c r="P56" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>19</v>
+      </c>
+      <c r="R56" t="s">
+        <v>22</v>
+      </c>
+      <c r="T56">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J57" t="s">
+        <v>75</v>
+      </c>
+      <c r="K57" t="s">
+        <v>19</v>
+      </c>
+      <c r="L57" t="s">
+        <v>76</v>
+      </c>
+      <c r="M57" t="s">
+        <v>16</v>
+      </c>
+      <c r="O57">
+        <v>2</v>
+      </c>
+      <c r="P57" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>19</v>
+      </c>
+      <c r="R57" t="s">
+        <v>23</v>
+      </c>
+      <c r="T57">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2975,7 +2994,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7990636-0CF9-6941-8EF6-80CF48D8BDA7}">
-  <dimension ref="J14:T34"/>
+  <dimension ref="J14:T36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="16" max="16" width="14.5" bestFit="1" customWidth="1"/>
@@ -3013,606 +3032,641 @@
       </c>
     </row>
     <row r="15" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
         <v>24</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="M15" t="s">
         <v>37</v>
       </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
         <v>38</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="2" t="s">
+      <c r="Q15" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" t="s">
         <v>47</v>
       </c>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2">
+      <c r="T15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>7</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="2" t="s">
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" t="s">
         <v>25</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M16" t="s">
         <v>37</v>
       </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2">
-        <v>1</v>
-      </c>
-      <c r="P16" s="2" t="s">
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16" t="s">
         <v>38</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="2" t="s">
+      <c r="Q16" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" t="s">
         <v>47</v>
       </c>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2">
+      <c r="T16">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J17" s="2" t="s">
+      <c r="J17" t="s">
         <v>8</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L17" s="2" t="s">
+      <c r="K17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L17" t="s">
         <v>24</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M17" t="s">
         <v>37</v>
       </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="s">
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17" t="s">
         <v>38</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R17" s="2" t="s">
+      <c r="Q17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R17" t="s">
         <v>47</v>
       </c>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2">
+      <c r="T17">
         <v>3</v>
       </c>
     </row>
     <row r="18" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J18" s="2" t="s">
+      <c r="J18" t="s">
         <v>9</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="K18" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M18" t="s">
         <v>37</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18" t="s">
         <v>38</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R18" s="2" t="s">
+      <c r="Q18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R18" t="s">
         <v>47</v>
       </c>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2">
+      <c r="T18">
         <v>4</v>
       </c>
     </row>
     <row r="19" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J19" s="2" t="s">
+      <c r="J19" t="s">
         <v>10</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="K19" t="s">
+        <v>19</v>
+      </c>
+      <c r="L19" t="s">
         <v>25</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" t="s">
         <v>37</v>
       </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2">
-        <v>1</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19" t="s">
         <v>38</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R19" s="2" t="s">
+      <c r="Q19" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" t="s">
         <v>47</v>
       </c>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2">
+      <c r="T19">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J20" s="2" t="s">
+      <c r="J20" t="s">
         <v>11</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="K20" t="s">
+        <v>19</v>
+      </c>
+      <c r="L20" t="s">
         <v>26</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="M20" t="s">
         <v>37</v>
       </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2">
-        <v>1</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20" t="s">
         <v>38</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R20" s="2" t="s">
+      <c r="Q20" t="s">
+        <v>18</v>
+      </c>
+      <c r="R20" t="s">
         <v>47</v>
       </c>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2">
+      <c r="T20">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J21" s="2" t="s">
+      <c r="J21" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="K21" t="s">
+        <v>18</v>
+      </c>
+      <c r="L21" t="s">
         <v>27</v>
       </c>
-      <c r="M21" s="2" t="s">
+      <c r="M21" t="s">
         <v>37</v>
       </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21" t="s">
         <v>38</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R21" s="2" t="s">
+      <c r="Q21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R21" t="s">
         <v>47</v>
       </c>
-      <c r="S21" s="2"/>
-      <c r="T21" s="2">
+      <c r="T21">
         <v>7</v>
       </c>
     </row>
     <row r="22" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J22" s="2" t="s">
+      <c r="J22" t="s">
         <v>13</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="K22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" t="s">
         <v>28</v>
       </c>
-      <c r="M22" s="2" t="s">
+      <c r="M22" t="s">
         <v>37</v>
       </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2">
-        <v>1</v>
-      </c>
-      <c r="P22" s="2" t="s">
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22" t="s">
         <v>38</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="Q22" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" t="s">
         <v>47</v>
       </c>
-      <c r="S22" s="2"/>
-      <c r="T22" s="2">
+      <c r="T22">
         <v>8</v>
       </c>
     </row>
     <row r="23" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J23" s="2" t="s">
+      <c r="J23" t="s">
         <v>14</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="K23" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" t="s">
         <v>27</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="M23" t="s">
         <v>37</v>
       </c>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2">
-        <v>1</v>
-      </c>
-      <c r="P23" s="2" t="s">
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23" t="s">
         <v>38</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R23" s="2" t="s">
+      <c r="Q23" t="s">
+        <v>18</v>
+      </c>
+      <c r="R23" t="s">
         <v>47</v>
       </c>
-      <c r="S23" s="2"/>
-      <c r="T23" s="2">
+      <c r="T23">
         <v>9</v>
       </c>
     </row>
     <row r="24" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>15</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="K24" t="s">
+        <v>19</v>
+      </c>
+      <c r="L24" t="s">
         <v>28</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" t="s">
         <v>37</v>
       </c>
-      <c r="O24" s="2">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24" t="s">
         <v>38</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R24" s="2" t="s">
+      <c r="Q24" t="s">
+        <v>18</v>
+      </c>
+      <c r="R24" t="s">
         <v>47</v>
       </c>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2">
+      <c r="T24">
         <v>10</v>
       </c>
     </row>
     <row r="25" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>52</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="K25" t="s">
         <v>20</v>
       </c>
-      <c r="L25" s="2" t="s">
+      <c r="L25" t="s">
         <v>56</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" t="s">
         <v>37</v>
       </c>
-      <c r="O25" s="2">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
         <v>38</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R25" s="2" t="s">
+      <c r="Q25" t="s">
+        <v>18</v>
+      </c>
+      <c r="R25" t="s">
         <v>47</v>
       </c>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2">
+      <c r="T25">
         <v>11</v>
       </c>
     </row>
     <row r="26" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>53</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K26" t="s">
         <v>20</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="L26" t="s">
         <v>57</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" t="s">
         <v>37</v>
       </c>
-      <c r="O26" s="2">
-        <v>1</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26">
+        <v>1</v>
+      </c>
+      <c r="P26" t="s">
         <v>38</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R26" s="2" t="s">
+      <c r="Q26" t="s">
+        <v>18</v>
+      </c>
+      <c r="R26" t="s">
         <v>47</v>
       </c>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2">
+      <c r="T26">
         <v>12</v>
       </c>
     </row>
     <row r="27" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>54</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K27" t="s">
         <v>20</v>
       </c>
-      <c r="L27" s="2" t="s">
+      <c r="L27" t="s">
         <v>58</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" t="s">
         <v>37</v>
       </c>
-      <c r="O27" s="2">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
         <v>38</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="Q27" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" t="s">
         <v>47</v>
       </c>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2">
+      <c r="T27">
         <v>13</v>
       </c>
     </row>
     <row r="28" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J28" s="2" t="s">
+      <c r="J28" t="s">
         <v>55</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="K28" t="s">
         <v>20</v>
       </c>
-      <c r="L28" s="2" t="s">
+      <c r="L28" t="s">
         <v>59</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" t="s">
         <v>37</v>
       </c>
-      <c r="O28" s="2">
-        <v>1</v>
-      </c>
-      <c r="P28" s="2" t="s">
+      <c r="O28">
+        <v>1</v>
+      </c>
+      <c r="P28" t="s">
         <v>38</v>
       </c>
-      <c r="Q28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R28" s="2" t="s">
+      <c r="Q28" t="s">
+        <v>18</v>
+      </c>
+      <c r="R28" t="s">
         <v>47</v>
       </c>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2">
+      <c r="T28">
         <v>14</v>
       </c>
     </row>
     <row r="29" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J29" s="2" t="s">
+      <c r="J29" t="s">
         <v>61</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L29" s="2" t="s">
+      <c r="K29" t="s">
+        <v>18</v>
+      </c>
+      <c r="L29" t="s">
         <v>62</v>
       </c>
-      <c r="M29" s="2" t="s">
+      <c r="M29" t="s">
         <v>37</v>
       </c>
-      <c r="O29" s="2">
-        <v>1</v>
-      </c>
-      <c r="P29" s="2" t="s">
+      <c r="O29">
+        <v>1</v>
+      </c>
+      <c r="P29" t="s">
         <v>38</v>
       </c>
-      <c r="Q29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R29" s="2" t="s">
+      <c r="Q29" t="s">
+        <v>18</v>
+      </c>
+      <c r="R29" t="s">
         <v>47</v>
       </c>
-      <c r="T29" s="2">
+      <c r="T29">
         <v>15</v>
       </c>
     </row>
     <row r="30" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J30" s="2" t="s">
+      <c r="J30" t="s">
         <v>63</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L30" s="2" t="s">
+      <c r="K30" t="s">
+        <v>18</v>
+      </c>
+      <c r="L30" t="s">
         <v>62</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="M30" t="s">
         <v>37</v>
       </c>
-      <c r="O30" s="2">
-        <v>1</v>
-      </c>
-      <c r="P30" s="2" t="s">
+      <c r="O30">
+        <v>1</v>
+      </c>
+      <c r="P30" t="s">
         <v>38</v>
       </c>
-      <c r="Q30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R30" s="2" t="s">
+      <c r="Q30" t="s">
+        <v>18</v>
+      </c>
+      <c r="R30" t="s">
         <v>47</v>
       </c>
-      <c r="T30" s="2">
+      <c r="T30">
         <v>16</v>
       </c>
     </row>
     <row r="31" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J31" s="2" t="s">
+      <c r="J31" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L31" s="2" t="s">
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" t="s">
         <v>62</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="M31" t="s">
         <v>37</v>
       </c>
-      <c r="O31" s="2">
-        <v>1</v>
-      </c>
-      <c r="P31" s="2" t="s">
+      <c r="O31">
+        <v>1</v>
+      </c>
+      <c r="P31" t="s">
         <v>38</v>
       </c>
-      <c r="Q31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R31" s="2" t="s">
+      <c r="Q31" t="s">
+        <v>18</v>
+      </c>
+      <c r="R31" t="s">
         <v>47</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31">
         <v>17</v>
       </c>
     </row>
     <row r="32" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J32" s="2" t="s">
+      <c r="J32" t="s">
         <v>65</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L32" s="2" t="s">
+      <c r="K32" t="s">
+        <v>19</v>
+      </c>
+      <c r="L32" t="s">
         <v>62</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" t="s">
         <v>37</v>
       </c>
-      <c r="O32" s="2">
-        <v>1</v>
-      </c>
-      <c r="P32" s="2" t="s">
+      <c r="O32">
+        <v>1</v>
+      </c>
+      <c r="P32" t="s">
         <v>38</v>
       </c>
-      <c r="Q32" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R32" s="2" t="s">
+      <c r="Q32" t="s">
+        <v>18</v>
+      </c>
+      <c r="R32" t="s">
         <v>47</v>
       </c>
-      <c r="T32" s="2">
+      <c r="T32">
         <v>18</v>
       </c>
     </row>
     <row r="33" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J33" s="2" t="s">
+      <c r="J33" t="s">
         <v>66</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="K33" t="s">
+        <v>19</v>
+      </c>
+      <c r="L33" t="s">
         <v>69</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="M33" t="s">
         <v>37</v>
       </c>
-      <c r="O33" s="2">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="s">
+      <c r="O33">
+        <v>1</v>
+      </c>
+      <c r="P33" t="s">
         <v>38</v>
       </c>
-      <c r="Q33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R33" s="2" t="s">
+      <c r="Q33" t="s">
+        <v>18</v>
+      </c>
+      <c r="R33" t="s">
         <v>47</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33">
         <v>19</v>
       </c>
     </row>
     <row r="34" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J34" s="2" t="s">
+      <c r="J34" t="s">
         <v>67</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="K34" t="s">
+        <v>19</v>
+      </c>
+      <c r="L34" t="s">
         <v>68</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" t="s">
         <v>37</v>
       </c>
-      <c r="O34" s="2">
-        <v>1</v>
-      </c>
-      <c r="P34" s="2" t="s">
+      <c r="O34">
+        <v>1</v>
+      </c>
+      <c r="P34" t="s">
         <v>38</v>
       </c>
-      <c r="Q34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R34" s="2" t="s">
+      <c r="Q34" t="s">
+        <v>18</v>
+      </c>
+      <c r="R34" t="s">
         <v>47</v>
       </c>
-      <c r="T34" s="2">
+      <c r="T34">
         <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J35" t="s">
+        <v>74</v>
+      </c>
+      <c r="K35" t="s">
+        <v>18</v>
+      </c>
+      <c r="L35" t="s">
+        <v>76</v>
+      </c>
+      <c r="M35" t="s">
+        <v>37</v>
+      </c>
+      <c r="O35">
+        <v>1</v>
+      </c>
+      <c r="P35" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" t="s">
+        <v>47</v>
+      </c>
+      <c r="T35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="10:20" x14ac:dyDescent="0.2">
+      <c r="J36" t="s">
+        <v>75</v>
+      </c>
+      <c r="K36" t="s">
+        <v>19</v>
+      </c>
+      <c r="L36" t="s">
+        <v>76</v>
+      </c>
+      <c r="M36" t="s">
+        <v>37</v>
+      </c>
+      <c r="O36">
+        <v>1</v>
+      </c>
+      <c r="P36" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>18</v>
+      </c>
+      <c r="R36" t="s">
+        <v>47</v>
+      </c>
+      <c r="T36">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -3660,34 +3714,31 @@
       </c>
     </row>
     <row r="15" spans="10:21" x14ac:dyDescent="0.2">
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>41</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" t="s">
         <v>23</v>
       </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15" t="s">
         <v>39</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2">
-        <v>1</v>
-      </c>
-      <c r="U15" s="2" t="s">
+      <c r="Q15" t="s">
+        <v>18</v>
+      </c>
+      <c r="R15" t="s">
+        <v>22</v>
+      </c>
+      <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3695,7 +3746,7 @@
       <c r="J16" t="s">
         <v>43</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" t="s">
         <v>20</v>
       </c>
       <c r="L16" t="s">
@@ -3704,13 +3755,13 @@
       <c r="O16">
         <v>1</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" t="s">
         <v>39</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R16" s="2" t="s">
+      <c r="Q16" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" t="s">
         <v>22</v>
       </c>
       <c r="T16">
@@ -3721,7 +3772,7 @@
       <c r="J17" t="s">
         <v>44</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K17" t="s">
         <v>20</v>
       </c>
       <c r="L17" t="s">
@@ -3730,13 +3781,13 @@
       <c r="O17">
         <v>1</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="P17" t="s">
         <v>39</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R17" s="2" t="s">
+      <c r="Q17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R17" t="s">
         <v>22</v>
       </c>
       <c r="T17">
@@ -3747,7 +3798,7 @@
       <c r="J18" t="s">
         <v>45</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="K18" t="s">
         <v>20</v>
       </c>
       <c r="L18" t="s">
@@ -3756,13 +3807,13 @@
       <c r="O18">
         <v>1</v>
       </c>
-      <c r="P18" s="2" t="s">
+      <c r="P18" t="s">
         <v>39</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R18" s="2" t="s">
+      <c r="Q18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R18" t="s">
         <v>22</v>
       </c>
       <c r="T18">
@@ -3773,7 +3824,7 @@
       <c r="J19" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" t="s">
         <v>20</v>
       </c>
       <c r="L19" t="s">
@@ -3782,13 +3833,13 @@
       <c r="O19">
         <v>1</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="P19" t="s">
         <v>39</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R19" s="2" t="s">
+      <c r="Q19" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" t="s">
         <v>22</v>
       </c>
       <c r="T19">
@@ -3799,7 +3850,7 @@
       <c r="J20" t="s">
         <v>43</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K20" t="s">
         <v>20</v>
       </c>
       <c r="L20" t="s">
@@ -3808,13 +3859,13 @@
       <c r="O20">
         <v>2</v>
       </c>
-      <c r="P20" s="2" t="s">
+      <c r="P20" t="s">
         <v>40</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R20" s="2" t="s">
+      <c r="Q20" t="s">
+        <v>18</v>
+      </c>
+      <c r="R20" t="s">
         <v>22</v>
       </c>
       <c r="T20">
@@ -3825,7 +3876,7 @@
       <c r="J21" t="s">
         <v>44</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" t="s">
         <v>20</v>
       </c>
       <c r="L21" t="s">
@@ -3834,13 +3885,13 @@
       <c r="O21">
         <v>2</v>
       </c>
-      <c r="P21" s="2" t="s">
+      <c r="P21" t="s">
         <v>40</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R21" s="2" t="s">
+      <c r="Q21" t="s">
+        <v>18</v>
+      </c>
+      <c r="R21" t="s">
         <v>22</v>
       </c>
       <c r="T21">
@@ -3851,7 +3902,7 @@
       <c r="J22" t="s">
         <v>45</v>
       </c>
-      <c r="K22" s="2" t="s">
+      <c r="K22" t="s">
         <v>20</v>
       </c>
       <c r="L22" t="s">
@@ -3860,13 +3911,13 @@
       <c r="O22">
         <v>2</v>
       </c>
-      <c r="P22" s="2" t="s">
+      <c r="P22" t="s">
         <v>40</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R22" s="2" t="s">
+      <c r="Q22" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" t="s">
         <v>22</v>
       </c>
       <c r="T22">
@@ -3877,7 +3928,7 @@
       <c r="J23" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="2" t="s">
+      <c r="K23" t="s">
         <v>20</v>
       </c>
       <c r="L23" t="s">
@@ -3886,13 +3937,13 @@
       <c r="O23">
         <v>2</v>
       </c>
-      <c r="P23" s="2" t="s">
+      <c r="P23" t="s">
         <v>40</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R23" s="2" t="s">
+      <c r="Q23" t="s">
+        <v>18</v>
+      </c>
+      <c r="R23" t="s">
         <v>22</v>
       </c>
       <c r="T23">
@@ -3900,122 +3951,118 @@
       </c>
     </row>
     <row r="24" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J24" s="2" t="s">
+      <c r="J24" t="s">
         <v>52</v>
       </c>
-      <c r="K24" s="2" t="s">
+      <c r="K24" t="s">
         <v>20</v>
       </c>
-      <c r="L24" s="2" t="s">
+      <c r="L24" t="s">
         <v>56</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" t="s">
         <v>60</v>
       </c>
-      <c r="O24" s="2">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="O24">
+        <v>1</v>
+      </c>
+      <c r="P24" t="s">
         <v>38</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R24" s="2" t="s">
+      <c r="Q24" t="s">
+        <v>18</v>
+      </c>
+      <c r="R24" t="s">
         <v>47</v>
       </c>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2">
+      <c r="T24">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J25" s="2" t="s">
+      <c r="J25" t="s">
         <v>53</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="K25" t="s">
         <v>20</v>
       </c>
-      <c r="L25" s="2" t="s">
+      <c r="L25" t="s">
         <v>57</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" t="s">
         <v>60</v>
       </c>
-      <c r="O25" s="2">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25" t="s">
         <v>38</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R25" s="2" t="s">
+      <c r="Q25" t="s">
+        <v>18</v>
+      </c>
+      <c r="R25" t="s">
         <v>47</v>
       </c>
-      <c r="S25" s="2"/>
-      <c r="T25" s="2">
+      <c r="T25">
         <v>25</v>
       </c>
     </row>
     <row r="26" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J26" s="2" t="s">
+      <c r="J26" t="s">
         <v>54</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K26" t="s">
         <v>20</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="L26" t="s">
         <v>58</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" t="s">
         <v>60</v>
       </c>
-      <c r="O26" s="2">
-        <v>1</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26">
+        <v>1</v>
+      </c>
+      <c r="P26" t="s">
         <v>38</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R26" s="2" t="s">
+      <c r="Q26" t="s">
+        <v>18</v>
+      </c>
+      <c r="R26" t="s">
         <v>47</v>
       </c>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2">
+      <c r="T26">
         <v>26</v>
       </c>
     </row>
     <row r="27" spans="10:20" x14ac:dyDescent="0.2">
-      <c r="J27" s="2" t="s">
+      <c r="J27" t="s">
         <v>55</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K27" t="s">
         <v>20</v>
       </c>
-      <c r="L27" s="2" t="s">
+      <c r="L27" t="s">
         <v>59</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" t="s">
         <v>60</v>
       </c>
-      <c r="O27" s="2">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
         <v>38</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="R27" s="2" t="s">
+      <c r="Q27" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" t="s">
         <v>47</v>
       </c>
-      <c r="S27" s="2"/>
-      <c r="T27" s="2">
+      <c r="T27">
         <v>27</v>
       </c>
     </row>

</xml_diff>